<commit_message>
Add dashboard displaying monthly patient count per unit and improve logging.
Screenshot: https://storage.googleapis.com/screenshot-production-us-central1/8c7417ff-25e3-4894-9a88-ca4d88413804/d2a27ba5-bcbf-48e4-ad52-da0db16f1132.jpg
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,12 +501,52 @@
           <t>teste 1</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Ribeirão</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>26/02/2025</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>26/02/2025</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Natália</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Dr. Arthur</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>teste 1</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Ribeirão</t>
         </is>

</xml_diff>

<commit_message>
User checkpoint: Update cirurgias.xlsx to address logo display issue.
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:AY4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,221 @@
           <t>unidade</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>total_foliculos</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>frente</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>densidade_scketh</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>coroa</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>scalpe</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>peninsula_direita</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>peninsula_esquerda</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>safira</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>punch</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>solucao_frente</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>solucao_coroa</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>solucao_xilo_frente</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>q1_area</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>q1_furos</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>q1_fios</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>q2_area</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>q2_furos</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>q2_fios</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>q3_area</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>q3_furos</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>q3_fios</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>q4_area</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>q4_furos</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>q4_fios</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>infiltracao</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>sedacao</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>sangramento</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>implante_secundario</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>transamin</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>tadalafila</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>diprospam</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>fumante</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>antecedentes</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>comentarios</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>q1_densidade</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>q2_densidade</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>q3_densidade</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>q4_densidade</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>q1_taxa_quebra</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>q2_taxa_quebra</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>q3_taxa_quebra</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>q4_taxa_quebra</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -509,6 +724,49 @@
           <t>Ribeirão</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -541,15 +799,261 @@
           <t>teste 1</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Ribeirão</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-02-27</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>26/02/2025</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Natália, Ana</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Dr. Arthur</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">arthur </t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>3200</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Ribeirão</t>
-        </is>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>834</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>148</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="n">
+        <v>100</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>10</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>100</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>25</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>9.999999999999998</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>40.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
User checkpoint: Add Excel file for storing surgery data for dashboard.
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY4"/>
+  <dimension ref="A1:AY5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -878,10 +878,8 @@
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G4" t="n">
+        <v>5</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -893,10 +891,8 @@
           <t xml:space="preserve">arthur </t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>3200</t>
-        </is>
+      <c r="J4" t="n">
+        <v>3200</v>
       </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
@@ -909,100 +905,62 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>0.85</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>834</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AF4" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
-      </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>148</t>
-        </is>
-      </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AJ4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="R4" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="S4" t="n">
+        <v>4</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="n">
+        <v>2</v>
+      </c>
+      <c r="V4" t="n">
+        <v>10</v>
+      </c>
+      <c r="W4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="X4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>100</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>90</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>834</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>250</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>148</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>2</v>
       </c>
       <c r="AK4" t="inlineStr">
         <is>
@@ -1054,6 +1012,203 @@
       </c>
       <c r="AY4" t="n">
         <v>40.8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-02-27</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>26/02/2025</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Natália, Ana</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Dr. Daniel</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Teste</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>3200</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>800</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>678</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>1290</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="n">
+        <v>80</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>48</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>65.21739130434783</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>125</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>16.66666666666666</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>14</v>
+      </c>
+      <c r="AY5" t="n">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
User checkpoint: Update cirurgias.xlsx to address dashboard display issues after data upload.
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY5"/>
+  <dimension ref="A1:AY6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1041,10 +1041,8 @@
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="G5" t="n">
+        <v>6</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1056,10 +1054,8 @@
           <t>Teste</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>3200</t>
-        </is>
+      <c r="J5" t="n">
+        <v>3200</v>
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
@@ -1072,92 +1068,58 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>0.85</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="R5" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="S5" t="n">
+        <v>5</v>
       </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>800</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>678</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>1500</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>1290</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>1500</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>900</t>
-        </is>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AJ5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="V5" t="n">
+        <v>10</v>
+      </c>
+      <c r="W5" t="n">
+        <v>800</v>
+      </c>
+      <c r="X5" t="n">
+        <v>678</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>25</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>23</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>1500</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>1290</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>12</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>1500</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>900</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>1</v>
       </c>
       <c r="AK5" t="inlineStr">
         <is>
@@ -1209,6 +1171,203 @@
       </c>
       <c r="AY5" t="n">
         <v>40</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-02-27</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>26/02/2025</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Aline</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Dr. Daniel</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Teste</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>3200</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
User checkpoint: Add Excel file to store surgery data for dashboard.
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY6"/>
+  <dimension ref="A1:AY7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1200,10 +1200,8 @@
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="G6" t="n">
+        <v>4</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -1215,10 +1213,8 @@
           <t>Teste</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>3200</t>
-        </is>
+      <c r="J6" t="n">
+        <v>3200</v>
       </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
@@ -1231,92 +1227,58 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>0.85</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="R6" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="S6" t="n">
+        <v>10</v>
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AI6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AJ6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="V6" t="n">
+        <v>10</v>
+      </c>
+      <c r="W6" t="n">
+        <v>10</v>
+      </c>
+      <c r="X6" t="n">
+        <v>10</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>10</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>3</v>
       </c>
       <c r="AK6" t="inlineStr">
         <is>
@@ -1368,6 +1330,243 @@
       </c>
       <c r="AY6" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-02-28</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>27/02/2025</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Aline, Natália</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Dr. Arthur</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Marcelo</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>1550</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>710</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>181</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>800</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>711</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>1450</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>1389</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>1510</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>1400</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>650</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>501</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AR7" t="n">
+        <v>12.6984126984127</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>14.64646464646465</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>17.15909090909091</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>10.31746031746032</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>11.125</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>4.206896551724137</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>7.284768211920534</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>22.92307692307692</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Add password-protected data deletion button to Dashboard.
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP2"/>
+  <dimension ref="A1:AP3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -676,15 +676,11 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="H2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -697,92 +693,58 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>0.85</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="Q2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="R2" t="n">
+        <v>5</v>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="U2" t="n">
+        <v>10</v>
+      </c>
+      <c r="V2" t="n">
+        <v>10</v>
+      </c>
+      <c r="W2" t="n">
+        <v>10</v>
+      </c>
+      <c r="X2" t="n">
+        <v>10</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>10</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>3</v>
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
@@ -811,6 +773,178 @@
       </c>
       <c r="AO2" t="inlineStr"/>
       <c r="AP2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-03-08</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>07/03/2025</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Oi</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Dr. Arthur</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Natália</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update cirurgias.xlsx
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP3"/>
+  <dimension ref="A1:BH4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -637,6 +637,96 @@
       <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>comentarios</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>extra_person_1</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>extra_person_2</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>bloqueio</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>bloqueio_seringas</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>bloqueio_comentarios</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>barba_furos</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>barba_fios</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>barba_comentarios</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>peitoral_furos</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>peitoral_fios</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>peitoral_comentarios</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>abdome_furos</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>abdome_fios</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>abdome_comentarios</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>dorso_furos</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>dorso_fios</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>dorso_comentarios</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>bloqueio_data</t>
         </is>
       </c>
     </row>
@@ -773,6 +863,24 @@
       </c>
       <c r="AO2" t="inlineStr"/>
       <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="inlineStr"/>
+      <c r="BA2" t="inlineStr"/>
+      <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr"/>
+      <c r="BE2" t="inlineStr"/>
+      <c r="BF2" t="inlineStr"/>
+      <c r="BG2" t="inlineStr"/>
+      <c r="BH2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -810,15 +918,11 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -831,92 +935,58 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>0.85</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="Q3" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="R3" t="n">
+        <v>3</v>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AF3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AI3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="U3" t="n">
+        <v>1</v>
+      </c>
+      <c r="V3" t="n">
+        <v>1</v>
+      </c>
+      <c r="W3" t="n">
+        <v>1</v>
+      </c>
+      <c r="X3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>3</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
@@ -945,6 +1015,222 @@
       </c>
       <c r="AO3" t="inlineStr"/>
       <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+      <c r="AZ3" t="inlineStr"/>
+      <c r="BA3" t="inlineStr"/>
+      <c r="BB3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr"/>
+      <c r="BE3" t="inlineStr"/>
+      <c r="BF3" t="inlineStr"/>
+      <c r="BG3" t="inlineStr"/>
+      <c r="BH3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-03-10</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>09/03/2025</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">arthur </t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Dr. Arthur</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Natália</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr"/>
+      <c r="AX4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr"/>
+      <c r="AZ4" t="inlineStr"/>
+      <c r="BA4" t="inlineStr"/>
+      <c r="BB4" t="inlineStr"/>
+      <c r="BC4" t="inlineStr"/>
+      <c r="BD4" t="inlineStr"/>
+      <c r="BE4" t="inlineStr"/>
+      <c r="BF4" t="inlineStr"/>
+      <c r="BG4" t="inlineStr"/>
+      <c r="BH4" t="inlineStr">
+        <is>
+          <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Create checkpoint: Application running perfectly.
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH4"/>
+  <dimension ref="A1:BH2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -733,51 +733,63 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-03-08</t>
+          <t>2025-03-10</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>07/03/2025</t>
+          <t>09/03/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Arthur</t>
+          <t>Carlos Eduardo Milani</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Ribeirão Preto</t>
+          <t>Rio de Janeiro</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Dr. Daniel</t>
+          <t>Dra. Ana Clara</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Natália</t>
+          <t>Mariana Moro, Mariana Silva, Assistente Extra, Aline  (extra), Natália  (extra)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+        <v>3414</v>
+      </c>
+      <c r="J2" t="n">
+        <v>2964</v>
+      </c>
+      <c r="K2" t="n">
+        <v>80</v>
+      </c>
+      <c r="L2" t="n">
+        <v>450</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>200</v>
+      </c>
+      <c r="O2" t="n">
+        <v>200</v>
+      </c>
       <c r="P2" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -787,87 +799,118 @@
         <v>0.85</v>
       </c>
       <c r="R2" t="n">
-        <v>5</v>
-      </c>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="S2" t="n">
+        <v>3</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
       <c r="U2" t="n">
-        <v>10</v>
+        <v>48</v>
       </c>
       <c r="V2" t="n">
-        <v>10</v>
+        <v>650</v>
       </c>
       <c r="W2" t="n">
-        <v>10</v>
+        <v>637</v>
       </c>
       <c r="X2" t="n">
-        <v>10</v>
+        <v>68</v>
       </c>
       <c r="Y2" t="n">
-        <v>10</v>
+        <v>1150</v>
       </c>
       <c r="Z2" t="n">
-        <v>10</v>
+        <v>1027</v>
       </c>
       <c r="AA2" t="n">
-        <v>10</v>
+        <v>64</v>
       </c>
       <c r="AB2" t="n">
-        <v>10</v>
+        <v>1200</v>
       </c>
       <c r="AC2" t="n">
-        <v>10</v>
+        <v>1100</v>
       </c>
       <c r="AD2" t="n">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="AE2" t="n">
-        <v>10</v>
+        <v>700</v>
       </c>
       <c r="AF2" t="n">
-        <v>10</v>
+        <v>650</v>
       </c>
       <c r="AG2" t="n">
         <v>1</v>
       </c>
       <c r="AH2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AI2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nega </t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fios de 2 e 3 comprimentos médios e grossos </t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aline </t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Natália </t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>Xilo sem vaso</t>
+        </is>
+      </c>
+      <c r="AT2" t="n">
         <v>3</v>
       </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>A dra aqui faz um bloqueio diferente uma seringa de 3 ml 1,5 de xilo e 1,5 de soro 
+E duas seringas  de 1,5 ropi e 1,5 de soro</t>
+        </is>
+      </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr"/>
@@ -880,355 +923,9 @@
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-03-08</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>07/03/2025</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Oi</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Ribeirão Preto</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Dr. Arthur</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Natália</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>5</v>
-      </c>
-      <c r="I3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="R3" t="n">
-        <v>3</v>
-      </c>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="n">
-        <v>1</v>
-      </c>
-      <c r="V3" t="n">
-        <v>1</v>
-      </c>
-      <c r="W3" t="n">
-        <v>1</v>
-      </c>
-      <c r="X3" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH3" t="n">
-        <v>2</v>
-      </c>
-      <c r="AI3" t="n">
-        <v>3</v>
-      </c>
-      <c r="AJ3" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AK3" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AL3" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AM3" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AN3" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr"/>
-      <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr"/>
-      <c r="AX3" t="inlineStr"/>
-      <c r="AY3" t="inlineStr"/>
-      <c r="AZ3" t="inlineStr"/>
-      <c r="BA3" t="inlineStr"/>
-      <c r="BB3" t="inlineStr"/>
-      <c r="BC3" t="inlineStr"/>
-      <c r="BD3" t="inlineStr"/>
-      <c r="BE3" t="inlineStr"/>
-      <c r="BF3" t="inlineStr"/>
-      <c r="BG3" t="inlineStr"/>
-      <c r="BH3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-03-10</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>09/03/2025</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">arthur </t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Ribeirão Preto</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Dr. Arthur</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Natália</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AF4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AJ4" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AK4" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AL4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AM4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AN4" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AO4" t="inlineStr"/>
-      <c r="AP4" t="inlineStr"/>
-      <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr"/>
-      <c r="AS4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AT4" t="inlineStr"/>
-      <c r="AU4" t="inlineStr"/>
-      <c r="AV4" t="inlineStr"/>
-      <c r="AW4" t="inlineStr"/>
-      <c r="AX4" t="inlineStr"/>
-      <c r="AY4" t="inlineStr"/>
-      <c r="AZ4" t="inlineStr"/>
-      <c r="BA4" t="inlineStr"/>
-      <c r="BB4" t="inlineStr"/>
-      <c r="BC4" t="inlineStr"/>
-      <c r="BD4" t="inlineStr"/>
-      <c r="BE4" t="inlineStr"/>
-      <c r="BF4" t="inlineStr"/>
-      <c r="BG4" t="inlineStr"/>
-      <c r="BH4" t="inlineStr">
-        <is>
-          <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+      <c r="BH2" t="inlineStr">
+        <is>
+          <t>{"tipo":"Xilo sem vaso","seringas":"3","comentarios":"A dra aqui faz um bloqueio diferente uma seringa de 3 ml 1,5 de xilo e 1,5 de soro \nE duas seringas  de 1,5 ropi e 1,5 de soro"}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Remove "Import Data" button from dashboard.
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH2"/>
+  <dimension ref="A1:BH3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -929,6 +929,174 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-03-06</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>05/03/2025</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Jonas Galatti Carbonera</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Dr. Daniel</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Aline, Natália, Ana, thamara (extra)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>3705</v>
+      </c>
+      <c r="J3" t="n">
+        <v>3705</v>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="R3" t="n">
+        <v>8</v>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="n">
+        <v>1</v>
+      </c>
+      <c r="U3" t="n">
+        <v>55</v>
+      </c>
+      <c r="V3" t="n">
+        <v>750</v>
+      </c>
+      <c r="W3" t="n">
+        <v>730</v>
+      </c>
+      <c r="X3" t="n">
+        <v>76</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>1250</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>1202</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>76</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>1200</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>1186</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>48</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>630</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>587</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>thamara</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+      <c r="AZ3" t="inlineStr"/>
+      <c r="BA3" t="inlineStr"/>
+      <c r="BB3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr"/>
+      <c r="BE3" t="inlineStr"/>
+      <c r="BF3" t="inlineStr"/>
+      <c r="BG3" t="inlineStr"/>
+      <c r="BH3" t="inlineStr">
+        <is>
+          <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Create backup of `cirurgias.xlsx` file.
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH4"/>
+  <dimension ref="A1:BH10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1273,6 +1273,1101 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-03-06</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>05/03/2025</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>adnan jamil el homoui</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Dr. Arthur</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Aline, Natália, Ana, thamara (extra)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3400</v>
+      </c>
+      <c r="J5" t="n">
+        <v>2850</v>
+      </c>
+      <c r="K5" t="n">
+        <v>100</v>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="n">
+        <v>310</v>
+      </c>
+      <c r="O5" t="n">
+        <v>239</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="R5" t="n">
+        <v>3</v>
+      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="n">
+        <v>-2</v>
+      </c>
+      <c r="U5" t="n">
+        <v>45</v>
+      </c>
+      <c r="V5" t="n">
+        <v>630</v>
+      </c>
+      <c r="W5" t="n">
+        <v>585</v>
+      </c>
+      <c r="X5" t="n">
+        <v>60</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>1120</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>1090</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>64</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>1060</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>53</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>750</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>665</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>has</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>thamara</t>
+        </is>
+      </c>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr"/>
+      <c r="AZ5" t="inlineStr"/>
+      <c r="BA5" t="inlineStr"/>
+      <c r="BB5" t="inlineStr"/>
+      <c r="BC5" t="inlineStr"/>
+      <c r="BD5" t="inlineStr"/>
+      <c r="BE5" t="inlineStr"/>
+      <c r="BF5" t="inlineStr"/>
+      <c r="BG5" t="inlineStr"/>
+      <c r="BH5" t="inlineStr">
+        <is>
+          <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-03-06</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>05/03/2025</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hygor Henrique Bonfante</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Dr. Arthur</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Aline, Natália, Ana, thamara (extra)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3572</v>
+      </c>
+      <c r="J6" t="n">
+        <v>3162</v>
+      </c>
+      <c r="K6" t="n">
+        <v>106</v>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="n">
+        <v>210</v>
+      </c>
+      <c r="O6" t="n">
+        <v>2</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="R6" t="n">
+        <v>5</v>
+      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="n">
+        <v>1</v>
+      </c>
+      <c r="U6" t="n">
+        <v>45</v>
+      </c>
+      <c r="V6" t="n">
+        <v>400</v>
+      </c>
+      <c r="W6" t="n">
+        <v>370</v>
+      </c>
+      <c r="X6" t="n">
+        <v>72</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>1450</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>1365</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>76</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>1200</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>1170</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>48</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>700</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>667</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>nega</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fio 2 e 3. Fios de médio comprimento e médio 
+</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>thamara</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr"/>
+      <c r="AZ6" t="inlineStr"/>
+      <c r="BA6" t="inlineStr"/>
+      <c r="BB6" t="inlineStr"/>
+      <c r="BC6" t="inlineStr"/>
+      <c r="BD6" t="inlineStr"/>
+      <c r="BE6" t="inlineStr"/>
+      <c r="BF6" t="inlineStr"/>
+      <c r="BG6" t="inlineStr"/>
+      <c r="BH6" t="inlineStr">
+        <is>
+          <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-03-13</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>12/03/2025</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Eduardo Roncaglia de Carvalho</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Dr. Daniel</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Aline, Natália, thamara (extra)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" t="n">
+        <v>3655</v>
+      </c>
+      <c r="J7" t="n">
+        <v>2610</v>
+      </c>
+      <c r="K7" t="n">
+        <v>105</v>
+      </c>
+      <c r="L7" t="n">
+        <v>840</v>
+      </c>
+      <c r="M7" t="n">
+        <v>200</v>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="R7" t="n">
+        <v>4</v>
+      </c>
+      <c r="S7" t="n">
+        <v>5</v>
+      </c>
+      <c r="T7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U7" t="n">
+        <v>49</v>
+      </c>
+      <c r="V7" t="n">
+        <v>630</v>
+      </c>
+      <c r="W7" t="n">
+        <v>585</v>
+      </c>
+      <c r="X7" t="n">
+        <v>81</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>1300</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>1249</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>72</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>1300</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>1217</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>48</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>670</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>604</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>nega</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fio 2  e 3 . Fios grossos  e médio . 
+</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>thamara</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr"/>
+      <c r="AU7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr"/>
+      <c r="AW7" t="inlineStr"/>
+      <c r="AX7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr"/>
+      <c r="AZ7" t="inlineStr"/>
+      <c r="BA7" t="inlineStr"/>
+      <c r="BB7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr"/>
+      <c r="BD7" t="inlineStr"/>
+      <c r="BE7" t="inlineStr"/>
+      <c r="BF7" t="inlineStr"/>
+      <c r="BG7" t="inlineStr"/>
+      <c r="BH7" t="inlineStr">
+        <is>
+          <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-03-10</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>09/03/2025</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Weslei Diego Pavini</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Dr. Arthur</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Ana, angelica  (extra), larissa (extra)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>5</v>
+      </c>
+      <c r="I8" t="n">
+        <v>3800</v>
+      </c>
+      <c r="J8" t="n">
+        <v>3560</v>
+      </c>
+      <c r="K8" t="n">
+        <v>76</v>
+      </c>
+      <c r="L8" t="n">
+        <v>240</v>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="n">
+        <v>100</v>
+      </c>
+      <c r="O8" t="n">
+        <v>98</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="R8" t="n">
+        <v>7</v>
+      </c>
+      <c r="S8" t="n">
+        <v>2</v>
+      </c>
+      <c r="T8" t="n">
+        <v>1</v>
+      </c>
+      <c r="U8" t="n">
+        <v>62</v>
+      </c>
+      <c r="V8" t="n">
+        <v>630</v>
+      </c>
+      <c r="W8" t="n">
+        <v>600</v>
+      </c>
+      <c r="X8" t="n">
+        <v>93</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>1350</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>1300</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>88</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>1708</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>1508</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>54</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>400</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>320</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">angelica </t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>larissa</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr"/>
+      <c r="AU8" t="inlineStr"/>
+      <c r="AV8" t="inlineStr"/>
+      <c r="AW8" t="inlineStr"/>
+      <c r="AX8" t="inlineStr"/>
+      <c r="AY8" t="inlineStr"/>
+      <c r="AZ8" t="inlineStr"/>
+      <c r="BA8" t="inlineStr"/>
+      <c r="BB8" t="inlineStr"/>
+      <c r="BC8" t="inlineStr"/>
+      <c r="BD8" t="inlineStr"/>
+      <c r="BE8" t="inlineStr"/>
+      <c r="BF8" t="inlineStr"/>
+      <c r="BG8" t="inlineStr"/>
+      <c r="BH8" t="inlineStr">
+        <is>
+          <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-03-07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06/03/2025</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maurício Ronaldo Ribeiro </t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Dr. Arthur</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Ana, angelica  (extra), larissa (extra)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3737</v>
+      </c>
+      <c r="J9" t="n">
+        <v>3737</v>
+      </c>
+      <c r="K9" t="n">
+        <v>80</v>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="R9" t="n">
+        <v>7</v>
+      </c>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="n">
+        <v>1</v>
+      </c>
+      <c r="U9" t="n">
+        <v>62</v>
+      </c>
+      <c r="V9" t="n">
+        <v>630</v>
+      </c>
+      <c r="W9" t="n">
+        <v>600</v>
+      </c>
+      <c r="X9" t="n">
+        <v>72</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>1470</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>1400</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>68</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>1470</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>1400</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>49</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>420</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>387</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> fio 1 e 2 Fios fino e longo.</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">angelica </t>
+        </is>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>larissa</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT9" t="inlineStr"/>
+      <c r="AU9" t="inlineStr"/>
+      <c r="AV9" t="inlineStr"/>
+      <c r="AW9" t="inlineStr"/>
+      <c r="AX9" t="inlineStr"/>
+      <c r="AY9" t="inlineStr"/>
+      <c r="AZ9" t="inlineStr"/>
+      <c r="BA9" t="inlineStr"/>
+      <c r="BB9" t="inlineStr"/>
+      <c r="BC9" t="inlineStr"/>
+      <c r="BD9" t="inlineStr"/>
+      <c r="BE9" t="inlineStr"/>
+      <c r="BF9" t="inlineStr"/>
+      <c r="BG9" t="inlineStr"/>
+      <c r="BH9" t="inlineStr">
+        <is>
+          <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025-03-11</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>10/03/2025</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>José Antônio Tonetto Neto</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Dr. Daniel</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Ana, angelica  (extra), larissa (extra)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3498</v>
+      </c>
+      <c r="J10" t="n">
+        <v>808</v>
+      </c>
+      <c r="K10" t="n">
+        <v>33</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M10" t="n">
+        <v>1190</v>
+      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="R10" t="n">
+        <v>2</v>
+      </c>
+      <c r="S10" t="n">
+        <v>7</v>
+      </c>
+      <c r="T10" t="n">
+        <v>1</v>
+      </c>
+      <c r="U10" t="n">
+        <v>64</v>
+      </c>
+      <c r="V10" t="n">
+        <v>700</v>
+      </c>
+      <c r="W10" t="n">
+        <v>668</v>
+      </c>
+      <c r="X10" t="n">
+        <v>76</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>1050</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>930</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>76</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>1300</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>1200</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>57</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>750</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>700</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>nega</t>
+        </is>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fio 1 e 2 Fios fino e longo.
+</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">angelica </t>
+        </is>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>larissa</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr"/>
+      <c r="AW10" t="inlineStr"/>
+      <c r="AX10" t="inlineStr"/>
+      <c r="AY10" t="inlineStr"/>
+      <c r="AZ10" t="inlineStr"/>
+      <c r="BA10" t="inlineStr"/>
+      <c r="BB10" t="inlineStr"/>
+      <c r="BC10" t="inlineStr"/>
+      <c r="BD10" t="inlineStr"/>
+      <c r="BE10" t="inlineStr"/>
+      <c r="BF10" t="inlineStr"/>
+      <c r="BG10" t="inlineStr"/>
+      <c r="BH10" t="inlineStr">
+        <is>
+          <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Remove Arthur and correct duplicated Douglas entries from the database.
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH9"/>
+  <dimension ref="A1:BH10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2169,6 +2169,208 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025-03-18</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>17/03/2025</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">arthur </t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Dr. Daniel</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Natália, Ana</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr"/>
+      <c r="AW10" t="inlineStr"/>
+      <c r="AX10" t="inlineStr"/>
+      <c r="AY10" t="inlineStr"/>
+      <c r="AZ10" t="inlineStr"/>
+      <c r="BA10" t="inlineStr"/>
+      <c r="BB10" t="inlineStr"/>
+      <c r="BC10" t="inlineStr"/>
+      <c r="BD10" t="inlineStr"/>
+      <c r="BE10" t="inlineStr"/>
+      <c r="BF10" t="inlineStr"/>
+      <c r="BG10" t="inlineStr"/>
+      <c r="BH10" t="inlineStr">
+        <is>
+          <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Reduce number of Douglas surgeries in cirurgias.xlsx; backup created.
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH10"/>
+  <dimension ref="A1:BH9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>adnan jamil el homoui</t>
+          <t>Hygor Henrique Bonfante</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1114,21 +1114,21 @@
         <v>5</v>
       </c>
       <c r="I4" t="n">
-        <v>3400</v>
+        <v>3572</v>
       </c>
       <c r="J4" t="n">
-        <v>2850</v>
+        <v>3162</v>
       </c>
       <c r="K4" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="O4" t="n">
-        <v>239</v>
+        <v>2</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -1139,56 +1139,56 @@
         <v>0.85</v>
       </c>
       <c r="R4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="U4" t="n">
         <v>45</v>
       </c>
       <c r="V4" t="n">
-        <v>630</v>
+        <v>400</v>
       </c>
       <c r="W4" t="n">
-        <v>585</v>
+        <v>370</v>
       </c>
       <c r="X4" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="Y4" t="n">
-        <v>1120</v>
+        <v>1450</v>
       </c>
       <c r="Z4" t="n">
-        <v>1090</v>
+        <v>1365</v>
       </c>
       <c r="AA4" t="n">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="AB4" t="n">
         <v>1200</v>
       </c>
       <c r="AC4" t="n">
-        <v>1060</v>
+        <v>1170</v>
       </c>
       <c r="AD4" t="n">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="AE4" t="n">
-        <v>750</v>
+        <v>700</v>
       </c>
       <c r="AF4" t="n">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="AG4" t="n">
         <v>1</v>
       </c>
       <c r="AH4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="AL4" t="inlineStr">
@@ -1217,10 +1217,15 @@
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>has</t>
-        </is>
-      </c>
-      <c r="AP4" t="inlineStr"/>
+          <t>nega</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fio 2 e 3. Fios de médio comprimento e médio 
+</t>
+        </is>
+      </c>
       <c r="AQ4" t="inlineStr">
         <is>
           <t>thamara</t>
@@ -1255,17 +1260,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-03-06</t>
+          <t>2025-03-13</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>05/03/2025</t>
+          <t>12/03/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hygor Henrique Bonfante</t>
+          <t>Eduardo Roncaglia de Carvalho</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1275,39 +1280,39 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Dr. Arthur</t>
+          <t>Dr. Daniel</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Aline, Natália, Ana, thamara (extra)</t>
+          <t>Aline, Natália, thamara (extra)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="H5" t="n">
         <v>5</v>
       </c>
       <c r="I5" t="n">
-        <v>3572</v>
+        <v>3655</v>
       </c>
       <c r="J5" t="n">
-        <v>3162</v>
+        <v>2610</v>
       </c>
       <c r="K5" t="n">
-        <v>106</v>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="n">
-        <v>210</v>
-      </c>
-      <c r="O5" t="n">
-        <v>2</v>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="L5" t="n">
+        <v>840</v>
+      </c>
+      <c r="M5" t="n">
+        <v>200</v>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1317,47 +1322,49 @@
         <v>0.85</v>
       </c>
       <c r="R5" t="n">
+        <v>4</v>
+      </c>
+      <c r="S5" t="n">
         <v>5</v>
       </c>
-      <c r="S5" t="inlineStr"/>
       <c r="T5" t="n">
         <v>1</v>
       </c>
       <c r="U5" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="V5" t="n">
-        <v>400</v>
+        <v>630</v>
       </c>
       <c r="W5" t="n">
-        <v>370</v>
+        <v>585</v>
       </c>
       <c r="X5" t="n">
+        <v>81</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>1300</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>1249</v>
+      </c>
+      <c r="AA5" t="n">
         <v>72</v>
       </c>
-      <c r="Y5" t="n">
-        <v>1450</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>1365</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>76</v>
-      </c>
       <c r="AB5" t="n">
-        <v>1200</v>
+        <v>1300</v>
       </c>
       <c r="AC5" t="n">
-        <v>1170</v>
+        <v>1217</v>
       </c>
       <c r="AD5" t="n">
         <v>48</v>
       </c>
       <c r="AE5" t="n">
-        <v>700</v>
+        <v>670</v>
       </c>
       <c r="AF5" t="n">
-        <v>667</v>
+        <v>604</v>
       </c>
       <c r="AG5" t="n">
         <v>1</v>
@@ -1366,7 +1373,7 @@
         <v>2</v>
       </c>
       <c r="AI5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
@@ -1400,7 +1407,7 @@
       </c>
       <c r="AP5" t="inlineStr">
         <is>
-          <t xml:space="preserve">fio 2 e 3. Fios de médio comprimento e médio 
+          <t xml:space="preserve">fio 2  e 3 . Fios grossos  e médio . 
 </t>
         </is>
       </c>
@@ -1438,17 +1445,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-03-13</t>
+          <t>2025-03-10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12/03/2025</t>
+          <t>09/03/2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Eduardo Roncaglia de Carvalho</t>
+          <t>Weslei Diego Pavini</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1458,39 +1465,41 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Dr. Daniel</t>
+          <t>Dr. Arthur</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Aline, Natália, thamara (extra)</t>
+          <t>Ana, angelica  (extra), larissa (extra)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="H6" t="n">
         <v>5</v>
       </c>
       <c r="I6" t="n">
-        <v>3655</v>
+        <v>3800</v>
       </c>
       <c r="J6" t="n">
-        <v>2610</v>
+        <v>3560</v>
       </c>
       <c r="K6" t="n">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="L6" t="n">
-        <v>840</v>
-      </c>
-      <c r="M6" t="n">
-        <v>200</v>
-      </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+        <v>240</v>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="n">
+        <v>100</v>
+      </c>
+      <c r="O6" t="n">
+        <v>98</v>
+      </c>
       <c r="P6" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1500,58 +1509,58 @@
         <v>0.85</v>
       </c>
       <c r="R6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
       </c>
       <c r="U6" t="n">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="V6" t="n">
         <v>630</v>
       </c>
       <c r="W6" t="n">
-        <v>585</v>
+        <v>600</v>
       </c>
       <c r="X6" t="n">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="Y6" t="n">
+        <v>1350</v>
+      </c>
+      <c r="Z6" t="n">
         <v>1300</v>
       </c>
-      <c r="Z6" t="n">
-        <v>1249</v>
-      </c>
       <c r="AA6" t="n">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="AB6" t="n">
-        <v>1300</v>
+        <v>1708</v>
       </c>
       <c r="AC6" t="n">
-        <v>1217</v>
+        <v>1508</v>
       </c>
       <c r="AD6" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="AE6" t="n">
-        <v>670</v>
+        <v>400</v>
       </c>
       <c r="AF6" t="n">
-        <v>604</v>
+        <v>320</v>
       </c>
       <c r="AG6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH6" t="n">
         <v>2</v>
       </c>
       <c r="AI6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
@@ -1578,23 +1587,18 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AO6" t="inlineStr">
-        <is>
-          <t>nega</t>
-        </is>
-      </c>
-      <c r="AP6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fio 2  e 3 . Fios grossos  e médio . 
-</t>
-        </is>
-      </c>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>thamara</t>
-        </is>
-      </c>
-      <c r="AR6" t="inlineStr"/>
+          <t xml:space="preserve">angelica </t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>larissa</t>
+        </is>
+      </c>
       <c r="AS6" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1623,17 +1627,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-03-10</t>
+          <t>2025-03-07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>09/03/2025</t>
+          <t>06/03/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Weslei Diego Pavini</t>
+          <t xml:space="preserve">Maurício Ronaldo Ribeiro </t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1657,27 +1661,21 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="I7" t="n">
-        <v>3800</v>
+        <v>3737</v>
       </c>
       <c r="J7" t="n">
-        <v>3560</v>
+        <v>3737</v>
       </c>
       <c r="K7" t="n">
-        <v>76</v>
-      </c>
-      <c r="L7" t="n">
-        <v>240</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="n">
-        <v>100</v>
-      </c>
-      <c r="O7" t="n">
-        <v>98</v>
-      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1689,9 +1687,7 @@
       <c r="R7" t="n">
         <v>7</v>
       </c>
-      <c r="S7" t="n">
-        <v>2</v>
-      </c>
+      <c r="S7" t="inlineStr"/>
       <c r="T7" t="n">
         <v>1</v>
       </c>
@@ -1705,37 +1701,37 @@
         <v>600</v>
       </c>
       <c r="X7" t="n">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="Y7" t="n">
-        <v>1350</v>
+        <v>1470</v>
       </c>
       <c r="Z7" t="n">
-        <v>1300</v>
+        <v>1400</v>
       </c>
       <c r="AA7" t="n">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="AB7" t="n">
-        <v>1708</v>
+        <v>1470</v>
       </c>
       <c r="AC7" t="n">
-        <v>1508</v>
+        <v>1400</v>
       </c>
       <c r="AD7" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="AE7" t="n">
-        <v>400</v>
+        <v>420</v>
       </c>
       <c r="AF7" t="n">
-        <v>320</v>
+        <v>387</v>
       </c>
       <c r="AG7" t="n">
         <v>2</v>
       </c>
       <c r="AH7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AI7" t="n">
         <v>2</v>
@@ -1766,7 +1762,11 @@
         </is>
       </c>
       <c r="AO7" t="inlineStr"/>
-      <c r="AP7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> fio 1 e 2 Fios fino e longo.</t>
+        </is>
+      </c>
       <c r="AQ7" t="inlineStr">
         <is>
           <t xml:space="preserve">angelica </t>
@@ -1805,17 +1805,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-03-07</t>
+          <t>2025-03-11</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06/03/2025</t>
+          <t>10/03/2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maurício Ronaldo Ribeiro </t>
+          <t>José Antônio Tonetto Neto</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Dr. Arthur</t>
+          <t>Dr. Daniel</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1842,16 +1842,20 @@
         <v>6.5</v>
       </c>
       <c r="I8" t="n">
-        <v>3737</v>
+        <v>3498</v>
       </c>
       <c r="J8" t="n">
-        <v>3737</v>
+        <v>808</v>
       </c>
       <c r="K8" t="n">
-        <v>80</v>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
+        <v>33</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1190</v>
+      </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
@@ -1860,63 +1864,65 @@
         </is>
       </c>
       <c r="Q8" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="R8" t="n">
+        <v>2</v>
+      </c>
+      <c r="S8" t="n">
         <v>7</v>
       </c>
-      <c r="S8" t="inlineStr"/>
       <c r="T8" t="n">
         <v>1</v>
       </c>
       <c r="U8" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="V8" t="n">
-        <v>630</v>
+        <v>700</v>
       </c>
       <c r="W8" t="n">
-        <v>600</v>
+        <v>668</v>
       </c>
       <c r="X8" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="Y8" t="n">
-        <v>1470</v>
+        <v>1050</v>
       </c>
       <c r="Z8" t="n">
-        <v>1400</v>
+        <v>930</v>
       </c>
       <c r="AA8" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="AB8" t="n">
-        <v>1470</v>
+        <v>1300</v>
       </c>
       <c r="AC8" t="n">
-        <v>1400</v>
+        <v>1200</v>
       </c>
       <c r="AD8" t="n">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="AE8" t="n">
-        <v>420</v>
+        <v>750</v>
       </c>
       <c r="AF8" t="n">
-        <v>387</v>
+        <v>700</v>
       </c>
       <c r="AG8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH8" t="n">
         <v>2</v>
-      </c>
-      <c r="AH8" t="n">
-        <v>3</v>
       </c>
       <c r="AI8" t="n">
         <v>2</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="AK8" t="inlineStr">
@@ -1939,10 +1945,15 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AO8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>nega</t>
+        </is>
+      </c>
       <c r="AP8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> fio 1 e 2 Fios fino e longo.</t>
+          <t xml:space="preserve">fio 1 e 2 Fios fino e longo.
+</t>
         </is>
       </c>
       <c r="AQ8" t="inlineStr">
@@ -1983,17 +1994,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-03-11</t>
+          <t>2025-03-18</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>10/03/2025</t>
+          <t>17/03/2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>José Antônio Tonetto Neto</t>
+          <t xml:space="preserve">arthur </t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2008,7 +2019,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Ana, angelica  (extra), larissa (extra)</t>
+          <t>Natália, Ana</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2017,105 +2028,95 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>6.5</v>
+        <v>5</v>
       </c>
       <c r="I9" t="n">
-        <v>3498</v>
-      </c>
-      <c r="J9" t="n">
-        <v>808</v>
-      </c>
-      <c r="K9" t="n">
-        <v>33</v>
-      </c>
-      <c r="L9" t="n">
-        <v>1500</v>
-      </c>
-      <c r="M9" t="n">
-        <v>1190</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="Q9" t="n">
-        <v>0.95</v>
+        <v>0.85</v>
       </c>
       <c r="R9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S9" t="n">
-        <v>7</v>
-      </c>
-      <c r="T9" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="T9" t="inlineStr"/>
       <c r="U9" t="n">
-        <v>64</v>
+        <v>3</v>
       </c>
       <c r="V9" t="n">
-        <v>700</v>
+        <v>3</v>
       </c>
       <c r="W9" t="n">
-        <v>668</v>
+        <v>33</v>
       </c>
       <c r="X9" t="n">
-        <v>76</v>
+        <v>3</v>
       </c>
       <c r="Y9" t="n">
-        <v>1050</v>
+        <v>3</v>
       </c>
       <c r="Z9" t="n">
-        <v>930</v>
+        <v>3</v>
       </c>
       <c r="AA9" t="n">
-        <v>76</v>
+        <v>3</v>
       </c>
       <c r="AB9" t="n">
-        <v>1300</v>
+        <v>3</v>
       </c>
       <c r="AC9" t="n">
-        <v>1200</v>
+        <v>3</v>
       </c>
       <c r="AD9" t="n">
-        <v>57</v>
+        <v>3</v>
       </c>
       <c r="AE9" t="n">
-        <v>750</v>
+        <v>3</v>
       </c>
       <c r="AF9" t="n">
-        <v>700</v>
+        <v>3</v>
       </c>
       <c r="AG9" t="n">
         <v>1</v>
       </c>
       <c r="AH9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AI9" t="n">
         <v>2</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="AK9" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
       <c r="AL9" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="AM9" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="AN9" t="inlineStr">
@@ -2123,27 +2124,10 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AO9" t="inlineStr">
-        <is>
-          <t>nega</t>
-        </is>
-      </c>
-      <c r="AP9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fio 1 e 2 Fios fino e longo.
-</t>
-        </is>
-      </c>
-      <c r="AQ9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">angelica </t>
-        </is>
-      </c>
-      <c r="AR9" t="inlineStr">
-        <is>
-          <t>larissa</t>
-        </is>
-      </c>
+      <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr"/>
+      <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2169,208 +2153,6 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2025-03-18</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>17/03/2025</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">arthur </t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Ribeirão Preto</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Dr. Daniel</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Natália, Ana</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>0.85</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="X10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="Y10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="Z10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AC10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AD10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AE10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AF10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AG10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AH10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AI10" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AJ10" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AK10" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AL10" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AM10" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AN10" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AO10" t="inlineStr"/>
-      <c r="AP10" t="inlineStr"/>
-      <c r="AQ10" t="inlineStr"/>
-      <c r="AR10" t="inlineStr"/>
-      <c r="AS10" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AT10" t="inlineStr"/>
-      <c r="AU10" t="inlineStr"/>
-      <c r="AV10" t="inlineStr"/>
-      <c r="AW10" t="inlineStr"/>
-      <c r="AX10" t="inlineStr"/>
-      <c r="AY10" t="inlineStr"/>
-      <c r="AZ10" t="inlineStr"/>
-      <c r="BA10" t="inlineStr"/>
-      <c r="BB10" t="inlineStr"/>
-      <c r="BC10" t="inlineStr"/>
-      <c r="BD10" t="inlineStr"/>
-      <c r="BE10" t="inlineStr"/>
-      <c r="BF10" t="inlineStr"/>
-      <c r="BG10" t="inlineStr"/>
-      <c r="BH10" t="inlineStr">
-        <is>
-          <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Add Mauricio's data and backup of surgeries data.
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH14"/>
+  <dimension ref="A1:BH16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -938,19 +938,21 @@
         <v>5</v>
       </c>
       <c r="I3" t="n">
+        <v>3400</v>
+      </c>
+      <c r="J3" t="n">
         <v>2850</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>100</v>
       </c>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
         <v>310</v>
       </c>
       <c r="O3" t="n">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -965,7 +967,7 @@
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="U3" t="n">
         <v>45</v>
@@ -1001,7 +1003,7 @@
         <v>750</v>
       </c>
       <c r="AF3" t="n">
-        <v>885</v>
+        <v>665</v>
       </c>
       <c r="AG3" t="n">
         <v>1</v>
@@ -1019,7 +1021,7 @@
       </c>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="AL3" t="inlineStr">
@@ -1039,7 +1041,7 @@
       </c>
       <c r="AO3" t="inlineStr">
         <is>
-          <t>hipertenso em uso de alodipina</t>
+          <t>has</t>
         </is>
       </c>
       <c r="AP3" t="inlineStr"/>
@@ -1087,7 +1089,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>adnan jamil el homoui</t>
+          <t>Hygor Henrique Bonfante</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1114,21 +1116,21 @@
         <v>5</v>
       </c>
       <c r="I4" t="n">
-        <v>3400</v>
+        <v>3572</v>
       </c>
       <c r="J4" t="n">
-        <v>2850</v>
+        <v>3162</v>
       </c>
       <c r="K4" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="O4" t="n">
-        <v>239</v>
+        <v>2</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -1139,56 +1141,56 @@
         <v>0.85</v>
       </c>
       <c r="R4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="U4" t="n">
         <v>45</v>
       </c>
       <c r="V4" t="n">
-        <v>630</v>
+        <v>400</v>
       </c>
       <c r="W4" t="n">
-        <v>585</v>
+        <v>370</v>
       </c>
       <c r="X4" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="Y4" t="n">
-        <v>1120</v>
+        <v>1450</v>
       </c>
       <c r="Z4" t="n">
-        <v>1090</v>
+        <v>1365</v>
       </c>
       <c r="AA4" t="n">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="AB4" t="n">
         <v>1200</v>
       </c>
       <c r="AC4" t="n">
-        <v>1060</v>
+        <v>1170</v>
       </c>
       <c r="AD4" t="n">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="AE4" t="n">
-        <v>750</v>
+        <v>700</v>
       </c>
       <c r="AF4" t="n">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="AG4" t="n">
         <v>1</v>
       </c>
       <c r="AH4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
@@ -1197,7 +1199,7 @@
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="AL4" t="inlineStr">
@@ -1217,10 +1219,15 @@
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>has</t>
-        </is>
-      </c>
-      <c r="AP4" t="inlineStr"/>
+          <t>nega</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fio 2 e 3. Fios de médio comprimento e médio 
+</t>
+        </is>
+      </c>
       <c r="AQ4" t="inlineStr">
         <is>
           <t>thamara</t>
@@ -1255,17 +1262,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-03-06</t>
+          <t>2025-03-13</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>05/03/2025</t>
+          <t>12/03/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hygor Henrique Bonfante</t>
+          <t>Eduardo Roncaglia de Carvalho</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1275,39 +1282,39 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Dr. Arthur</t>
+          <t>Dr. Daniel</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Aline, Natália, Ana, thamara (extra)</t>
+          <t>Aline, Natália, thamara (extra)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="H5" t="n">
         <v>5</v>
       </c>
       <c r="I5" t="n">
-        <v>3572</v>
+        <v>3655</v>
       </c>
       <c r="J5" t="n">
-        <v>3162</v>
+        <v>2610</v>
       </c>
       <c r="K5" t="n">
-        <v>106</v>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="n">
-        <v>210</v>
-      </c>
-      <c r="O5" t="n">
-        <v>2</v>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="L5" t="n">
+        <v>840</v>
+      </c>
+      <c r="M5" t="n">
+        <v>200</v>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1317,47 +1324,49 @@
         <v>0.85</v>
       </c>
       <c r="R5" t="n">
+        <v>4</v>
+      </c>
+      <c r="S5" t="n">
         <v>5</v>
       </c>
-      <c r="S5" t="inlineStr"/>
       <c r="T5" t="n">
         <v>1</v>
       </c>
       <c r="U5" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="V5" t="n">
-        <v>400</v>
+        <v>630</v>
       </c>
       <c r="W5" t="n">
-        <v>370</v>
+        <v>585</v>
       </c>
       <c r="X5" t="n">
+        <v>81</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>1300</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>1249</v>
+      </c>
+      <c r="AA5" t="n">
         <v>72</v>
       </c>
-      <c r="Y5" t="n">
-        <v>1450</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>1365</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>76</v>
-      </c>
       <c r="AB5" t="n">
-        <v>1200</v>
+        <v>1300</v>
       </c>
       <c r="AC5" t="n">
-        <v>1170</v>
+        <v>1217</v>
       </c>
       <c r="AD5" t="n">
         <v>48</v>
       </c>
       <c r="AE5" t="n">
-        <v>700</v>
+        <v>670</v>
       </c>
       <c r="AF5" t="n">
-        <v>667</v>
+        <v>604</v>
       </c>
       <c r="AG5" t="n">
         <v>1</v>
@@ -1366,7 +1375,7 @@
         <v>2</v>
       </c>
       <c r="AI5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
@@ -1400,7 +1409,7 @@
       </c>
       <c r="AP5" t="inlineStr">
         <is>
-          <t xml:space="preserve">fio 2 e 3. Fios de médio comprimento e médio 
+          <t xml:space="preserve">fio 2  e 3 . Fios grossos  e médio . 
 </t>
         </is>
       </c>
@@ -1438,17 +1447,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-03-13</t>
+          <t>2025-03-10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12/03/2025</t>
+          <t>09/03/2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Eduardo Roncaglia de Carvalho</t>
+          <t>Weslei Diego Pavini</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1458,39 +1467,41 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Dr. Daniel</t>
+          <t>Dr. Arthur</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Aline, Natália, thamara (extra)</t>
+          <t>Ana, angelica  (extra), larissa (extra)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="H6" t="n">
         <v>5</v>
       </c>
       <c r="I6" t="n">
-        <v>3655</v>
+        <v>3800</v>
       </c>
       <c r="J6" t="n">
-        <v>2610</v>
+        <v>3560</v>
       </c>
       <c r="K6" t="n">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="L6" t="n">
-        <v>840</v>
-      </c>
-      <c r="M6" t="n">
-        <v>200</v>
-      </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+        <v>240</v>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="n">
+        <v>100</v>
+      </c>
+      <c r="O6" t="n">
+        <v>98</v>
+      </c>
       <c r="P6" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1500,58 +1511,58 @@
         <v>0.85</v>
       </c>
       <c r="R6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
       </c>
       <c r="U6" t="n">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="V6" t="n">
         <v>630</v>
       </c>
       <c r="W6" t="n">
-        <v>585</v>
+        <v>600</v>
       </c>
       <c r="X6" t="n">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="Y6" t="n">
+        <v>1350</v>
+      </c>
+      <c r="Z6" t="n">
         <v>1300</v>
       </c>
-      <c r="Z6" t="n">
-        <v>1249</v>
-      </c>
       <c r="AA6" t="n">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="AB6" t="n">
-        <v>1300</v>
+        <v>1708</v>
       </c>
       <c r="AC6" t="n">
-        <v>1217</v>
+        <v>1508</v>
       </c>
       <c r="AD6" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="AE6" t="n">
-        <v>670</v>
+        <v>400</v>
       </c>
       <c r="AF6" t="n">
-        <v>604</v>
+        <v>320</v>
       </c>
       <c r="AG6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH6" t="n">
         <v>2</v>
       </c>
       <c r="AI6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
@@ -1578,23 +1589,18 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AO6" t="inlineStr">
-        <is>
-          <t>nega</t>
-        </is>
-      </c>
-      <c r="AP6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fio 2  e 3 . Fios grossos  e médio . 
-</t>
-        </is>
-      </c>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>thamara</t>
-        </is>
-      </c>
-      <c r="AR6" t="inlineStr"/>
+          <t xml:space="preserve">angelica </t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>larissa</t>
+        </is>
+      </c>
       <c r="AS6" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1623,17 +1629,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-03-10</t>
+          <t>2025-03-07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>09/03/2025</t>
+          <t>06/03/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Weslei Diego Pavini</t>
+          <t xml:space="preserve">Maurício Ronaldo Ribeiro </t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1657,27 +1663,21 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="I7" t="n">
-        <v>3800</v>
+        <v>3737</v>
       </c>
       <c r="J7" t="n">
-        <v>3560</v>
+        <v>3737</v>
       </c>
       <c r="K7" t="n">
-        <v>76</v>
-      </c>
-      <c r="L7" t="n">
-        <v>240</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="n">
-        <v>100</v>
-      </c>
-      <c r="O7" t="n">
-        <v>98</v>
-      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1689,9 +1689,7 @@
       <c r="R7" t="n">
         <v>7</v>
       </c>
-      <c r="S7" t="n">
-        <v>2</v>
-      </c>
+      <c r="S7" t="inlineStr"/>
       <c r="T7" t="n">
         <v>1</v>
       </c>
@@ -1705,37 +1703,37 @@
         <v>600</v>
       </c>
       <c r="X7" t="n">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="Y7" t="n">
-        <v>1350</v>
+        <v>1470</v>
       </c>
       <c r="Z7" t="n">
-        <v>1300</v>
+        <v>1400</v>
       </c>
       <c r="AA7" t="n">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="AB7" t="n">
-        <v>1708</v>
+        <v>1470</v>
       </c>
       <c r="AC7" t="n">
-        <v>1508</v>
+        <v>1400</v>
       </c>
       <c r="AD7" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="AE7" t="n">
-        <v>400</v>
+        <v>420</v>
       </c>
       <c r="AF7" t="n">
-        <v>320</v>
+        <v>387</v>
       </c>
       <c r="AG7" t="n">
         <v>2</v>
       </c>
       <c r="AH7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AI7" t="n">
         <v>2</v>
@@ -1766,7 +1764,11 @@
         </is>
       </c>
       <c r="AO7" t="inlineStr"/>
-      <c r="AP7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> fio 1 e 2 Fios fino e longo.</t>
+        </is>
+      </c>
       <c r="AQ7" t="inlineStr">
         <is>
           <t xml:space="preserve">angelica </t>
@@ -1805,17 +1807,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-03-07</t>
+          <t>2025-03-11</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06/03/2025</t>
+          <t>10/03/2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maurício Ronaldo Ribeiro </t>
+          <t>José Antônio Tonetto Neto</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1825,7 +1827,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Dr. Arthur</t>
+          <t>Dr. Daniel</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1842,16 +1844,20 @@
         <v>6.5</v>
       </c>
       <c r="I8" t="n">
-        <v>3737</v>
+        <v>3498</v>
       </c>
       <c r="J8" t="n">
-        <v>3737</v>
+        <v>808</v>
       </c>
       <c r="K8" t="n">
-        <v>80</v>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
+        <v>33</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1190</v>
+      </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
@@ -1860,63 +1866,65 @@
         </is>
       </c>
       <c r="Q8" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="R8" t="n">
+        <v>2</v>
+      </c>
+      <c r="S8" t="n">
         <v>7</v>
       </c>
-      <c r="S8" t="inlineStr"/>
       <c r="T8" t="n">
         <v>1</v>
       </c>
       <c r="U8" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="V8" t="n">
-        <v>630</v>
+        <v>700</v>
       </c>
       <c r="W8" t="n">
-        <v>600</v>
+        <v>668</v>
       </c>
       <c r="X8" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="Y8" t="n">
-        <v>1470</v>
+        <v>1050</v>
       </c>
       <c r="Z8" t="n">
-        <v>1400</v>
+        <v>930</v>
       </c>
       <c r="AA8" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="AB8" t="n">
-        <v>1470</v>
+        <v>1300</v>
       </c>
       <c r="AC8" t="n">
-        <v>1400</v>
+        <v>1200</v>
       </c>
       <c r="AD8" t="n">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="AE8" t="n">
-        <v>420</v>
+        <v>750</v>
       </c>
       <c r="AF8" t="n">
-        <v>387</v>
+        <v>700</v>
       </c>
       <c r="AG8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH8" t="n">
         <v>2</v>
-      </c>
-      <c r="AH8" t="n">
-        <v>3</v>
       </c>
       <c r="AI8" t="n">
         <v>2</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="AK8" t="inlineStr">
@@ -1939,10 +1947,15 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AO8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>nega</t>
+        </is>
+      </c>
       <c r="AP8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> fio 1 e 2 Fios fino e longo.</t>
+          <t xml:space="preserve">fio 1 e 2 Fios fino e longo.
+</t>
         </is>
       </c>
       <c r="AQ8" t="inlineStr">
@@ -1993,7 +2006,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>José Antônio Tonetto Neto</t>
+          <t xml:space="preserve">Douglas Rodrigues Costa </t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2013,26 +2026,26 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="H9" t="n">
         <v>6.5</v>
       </c>
       <c r="I9" t="n">
-        <v>3498</v>
+        <v>4000</v>
       </c>
       <c r="J9" t="n">
-        <v>808</v>
+        <v>2710</v>
       </c>
       <c r="K9" t="n">
-        <v>33</v>
+        <v>99</v>
       </c>
       <c r="L9" t="n">
-        <v>1500</v>
+        <v>773</v>
       </c>
       <c r="M9" t="n">
-        <v>1190</v>
+        <v>517</v>
       </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
@@ -2045,7 +2058,7 @@
         <v>0.95</v>
       </c>
       <c r="R9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="S9" t="n">
         <v>7</v>
@@ -2054,60 +2067,60 @@
         <v>1</v>
       </c>
       <c r="U9" t="n">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="V9" t="n">
-        <v>700</v>
+        <v>450</v>
       </c>
       <c r="W9" t="n">
-        <v>668</v>
+        <v>360</v>
       </c>
       <c r="X9" t="n">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="Y9" t="n">
-        <v>1050</v>
+        <v>1700</v>
       </c>
       <c r="Z9" t="n">
-        <v>930</v>
+        <v>1590</v>
       </c>
       <c r="AA9" t="n">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="AB9" t="n">
-        <v>1300</v>
+        <v>1650</v>
       </c>
       <c r="AC9" t="n">
-        <v>1200</v>
+        <v>1544</v>
       </c>
       <c r="AD9" t="n">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="AE9" t="n">
-        <v>750</v>
+        <v>600</v>
       </c>
       <c r="AF9" t="n">
-        <v>700</v>
+        <v>503</v>
       </c>
       <c r="AG9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH9" t="n">
         <v>2</v>
       </c>
       <c r="AI9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="AK9" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
       <c r="AL9" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2128,12 +2141,7 @@
           <t>nega</t>
         </is>
       </c>
-      <c r="AP9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fio 1 e 2 Fios fino e longo.
-</t>
-        </is>
-      </c>
+      <c r="AP9" t="inlineStr"/>
       <c r="AQ9" t="inlineStr">
         <is>
           <t xml:space="preserve">angelica </t>
@@ -2172,17 +2180,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-03-11</t>
+          <t>2025-03-12</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10/03/2025</t>
+          <t>11/03/2025</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Douglas Rodrigues Costa </t>
+          <t xml:space="preserve">Pedro Rafael de Almeida Picaccio </t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2206,77 +2214,75 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="I10" t="n">
-        <v>4000</v>
+        <v>4222</v>
       </c>
       <c r="J10" t="n">
-        <v>2710</v>
+        <v>3872</v>
       </c>
       <c r="K10" t="n">
-        <v>99</v>
-      </c>
-      <c r="L10" t="n">
-        <v>773</v>
-      </c>
-      <c r="M10" t="n">
-        <v>517</v>
-      </c>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+        <v>108</v>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="n">
+        <v>180</v>
+      </c>
+      <c r="O10" t="n">
+        <v>170</v>
+      </c>
       <c r="P10" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
       <c r="Q10" t="n">
-        <v>0.95</v>
+        <v>0.85</v>
       </c>
       <c r="R10" t="n">
-        <v>6</v>
-      </c>
-      <c r="S10" t="n">
-        <v>7</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="S10" t="inlineStr"/>
       <c r="T10" t="n">
         <v>1</v>
       </c>
       <c r="U10" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="V10" t="n">
-        <v>450</v>
+        <v>700</v>
       </c>
       <c r="W10" t="n">
-        <v>360</v>
+        <v>647</v>
       </c>
       <c r="X10" t="n">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="Y10" t="n">
-        <v>1700</v>
+        <v>1640</v>
       </c>
       <c r="Z10" t="n">
-        <v>1590</v>
+        <v>1575</v>
       </c>
       <c r="AA10" t="n">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="AB10" t="n">
         <v>1650</v>
       </c>
       <c r="AC10" t="n">
-        <v>1544</v>
+        <v>1600</v>
       </c>
       <c r="AD10" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="AE10" t="n">
-        <v>600</v>
+        <v>459</v>
       </c>
       <c r="AF10" t="n">
-        <v>503</v>
+        <v>400</v>
       </c>
       <c r="AG10" t="n">
         <v>2</v>
@@ -2299,7 +2305,7 @@
       </c>
       <c r="AL10" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="AM10" t="inlineStr">
@@ -2317,7 +2323,11 @@
           <t>nega</t>
         </is>
       </c>
-      <c r="AP10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>io 1 e 2 Fios finos e curtos</t>
+        </is>
+      </c>
       <c r="AQ10" t="inlineStr">
         <is>
           <t xml:space="preserve">angelica </t>
@@ -2366,7 +2376,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pedro Rafael de Almeida Picaccio </t>
+          <t xml:space="preserve">Rodolfo Carola </t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2376,7 +2386,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Dr. Daniel</t>
+          <t>Dr. Arthur</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -2386,79 +2396,79 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="I11" t="n">
-        <v>4222</v>
+        <v>3630</v>
       </c>
       <c r="J11" t="n">
-        <v>3872</v>
+        <v>3464</v>
       </c>
       <c r="K11" t="n">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
-        <v>180</v>
+        <v>85</v>
       </c>
       <c r="O11" t="n">
-        <v>170</v>
+        <v>81</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="Q11" t="n">
         <v>0.85</v>
       </c>
       <c r="R11" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="n">
         <v>1</v>
       </c>
       <c r="U11" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="V11" t="n">
-        <v>700</v>
+        <v>500</v>
       </c>
       <c r="W11" t="n">
-        <v>647</v>
+        <v>433</v>
       </c>
       <c r="X11" t="n">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="Y11" t="n">
-        <v>1640</v>
+        <v>1550</v>
       </c>
       <c r="Z11" t="n">
-        <v>1575</v>
+        <v>1450</v>
       </c>
       <c r="AA11" t="n">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="AB11" t="n">
-        <v>1650</v>
+        <v>1300</v>
       </c>
       <c r="AC11" t="n">
-        <v>1600</v>
+        <v>1210</v>
       </c>
       <c r="AD11" t="n">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="AE11" t="n">
-        <v>459</v>
+        <v>600</v>
       </c>
       <c r="AF11" t="n">
-        <v>400</v>
+        <v>537</v>
       </c>
       <c r="AG11" t="n">
         <v>2</v>
@@ -2467,7 +2477,7 @@
         <v>2</v>
       </c>
       <c r="AI11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
@@ -2476,14 +2486,14 @@
       </c>
       <c r="AK11" t="inlineStr">
         <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="AL11" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
       <c r="AM11" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2501,7 +2511,7 @@
       </c>
       <c r="AP11" t="inlineStr">
         <is>
-          <t>io 1 e 2 Fios finos e curtos</t>
+          <t>fio 1 e 2 Fios de espessura média e comprimento médio</t>
         </is>
       </c>
       <c r="AQ11" t="inlineStr">
@@ -2542,17 +2552,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025-03-12</t>
+          <t>2025-03-13</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>11/03/2025</t>
+          <t>12/03/2025</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rodolfo Carola </t>
+          <t>Alan Ribeiro de Paula</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2562,7 +2572,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Dr. Arthur</t>
+          <t>Dr. Daniel</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -2576,84 +2586,86 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="I12" t="n">
-        <v>3630</v>
+        <v>3710</v>
       </c>
       <c r="J12" t="n">
-        <v>3464</v>
+        <v>3100</v>
       </c>
       <c r="K12" t="n">
-        <v>123</v>
-      </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="n">
-        <v>85</v>
-      </c>
-      <c r="O12" t="n">
-        <v>81</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="L12" t="n">
+        <v>425</v>
+      </c>
+      <c r="M12" t="n">
+        <v>185</v>
+      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="Q12" t="n">
         <v>0.85</v>
       </c>
       <c r="R12" t="n">
-        <v>5</v>
-      </c>
-      <c r="S12" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="S12" t="n">
+        <v>6</v>
+      </c>
       <c r="T12" t="n">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="U12" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V12" t="n">
+        <v>700</v>
+      </c>
+      <c r="W12" t="n">
+        <v>662</v>
+      </c>
+      <c r="X12" t="n">
+        <v>76</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>1420</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>1378</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>76</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>1430</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>1200</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>52</v>
+      </c>
+      <c r="AE12" t="n">
         <v>500</v>
       </c>
-      <c r="W12" t="n">
-        <v>433</v>
-      </c>
-      <c r="X12" t="n">
-        <v>90</v>
-      </c>
-      <c r="Y12" t="n">
-        <v>1550</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>1450</v>
-      </c>
-      <c r="AA12" t="n">
-        <v>93</v>
-      </c>
-      <c r="AB12" t="n">
-        <v>1300</v>
-      </c>
-      <c r="AC12" t="n">
-        <v>1210</v>
-      </c>
-      <c r="AD12" t="n">
-        <v>68</v>
-      </c>
-      <c r="AE12" t="n">
-        <v>600</v>
-      </c>
       <c r="AF12" t="n">
-        <v>537</v>
+        <v>470</v>
       </c>
       <c r="AG12" t="n">
         <v>2</v>
       </c>
       <c r="AH12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AI12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
@@ -2662,12 +2674,12 @@
       </c>
       <c r="AK12" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="AL12" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="AM12" t="inlineStr">
@@ -2687,7 +2699,8 @@
       </c>
       <c r="AP12" t="inlineStr">
         <is>
-          <t>fio 1 e 2 Fios de espessura média e comprimento médio</t>
+          <t xml:space="preserve">fio 1 e 2 Fios de espessura grossa e comprimento longo.
+</t>
         </is>
       </c>
       <c r="AQ12" t="inlineStr">
@@ -2738,7 +2751,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Alan Ribeiro de Paula</t>
+          <t xml:space="preserve">Lucas Colleoni Ruaro </t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2758,26 +2771,26 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="H13" t="n">
         <v>6</v>
       </c>
       <c r="I13" t="n">
-        <v>3710</v>
+        <v>3800</v>
       </c>
       <c r="J13" t="n">
-        <v>3100</v>
+        <v>2505</v>
       </c>
       <c r="K13" t="n">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="L13" t="n">
-        <v>425</v>
+        <v>1105</v>
       </c>
       <c r="M13" t="n">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
@@ -2793,52 +2806,52 @@
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="T13" t="n">
-        <v>-3</v>
+        <v>1</v>
       </c>
       <c r="U13" t="n">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="V13" t="n">
         <v>700</v>
       </c>
       <c r="W13" t="n">
-        <v>662</v>
+        <v>400</v>
       </c>
       <c r="X13" t="n">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="Y13" t="n">
-        <v>1420</v>
+        <v>1750</v>
       </c>
       <c r="Z13" t="n">
-        <v>1378</v>
+        <v>1500</v>
       </c>
       <c r="AA13" t="n">
-        <v>76</v>
+        <v>114</v>
       </c>
       <c r="AB13" t="n">
-        <v>1430</v>
+        <v>1500</v>
       </c>
       <c r="AC13" t="n">
-        <v>1200</v>
+        <v>1450</v>
       </c>
       <c r="AD13" t="n">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="AE13" t="n">
         <v>500</v>
       </c>
       <c r="AF13" t="n">
-        <v>470</v>
+        <v>450</v>
       </c>
       <c r="AG13" t="n">
         <v>2</v>
       </c>
       <c r="AH13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI13" t="n">
         <v>3</v>
@@ -2870,15 +2883,11 @@
       </c>
       <c r="AO13" t="inlineStr">
         <is>
-          <t>nega</t>
-        </is>
-      </c>
-      <c r="AP13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fio 1 e 2 Fios de espessura grossa e comprimento longo.
+          <t xml:space="preserve">fio 1 e 2 Fios de espessura fina e comprimento curto.
 </t>
         </is>
       </c>
+      <c r="AP13" t="inlineStr"/>
       <c r="AQ13" t="inlineStr">
         <is>
           <t xml:space="preserve">angelica </t>
@@ -2917,17 +2926,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2025-03-13</t>
+          <t>2025-03-14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>12/03/2025</t>
+          <t>13/03/2025</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lucas Colleoni Ruaro </t>
+          <t>Lucas Evandro de Melo</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2951,23 +2960,19 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I14" t="n">
-        <v>3800</v>
+        <v>4070</v>
       </c>
       <c r="J14" t="n">
-        <v>2505</v>
+        <v>4070</v>
       </c>
       <c r="K14" t="n">
-        <v>106</v>
-      </c>
-      <c r="L14" t="n">
-        <v>1105</v>
-      </c>
-      <c r="M14" t="n">
-        <v>190</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
@@ -2979,55 +2984,53 @@
         <v>0.85</v>
       </c>
       <c r="R14" t="n">
-        <v>7</v>
-      </c>
-      <c r="S14" t="n">
-        <v>1</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="S14" t="inlineStr"/>
       <c r="T14" t="n">
         <v>1</v>
       </c>
       <c r="U14" t="n">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="V14" t="n">
-        <v>700</v>
+        <v>600</v>
       </c>
       <c r="W14" t="n">
-        <v>400</v>
+        <v>550</v>
       </c>
       <c r="X14" t="n">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="Y14" t="n">
-        <v>1750</v>
+        <v>1600</v>
       </c>
       <c r="Z14" t="n">
+        <v>1550</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>96</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>1700</v>
+      </c>
+      <c r="AC14" t="n">
         <v>1500</v>
       </c>
-      <c r="AA14" t="n">
-        <v>114</v>
-      </c>
-      <c r="AB14" t="n">
-        <v>1500</v>
-      </c>
-      <c r="AC14" t="n">
-        <v>1450</v>
-      </c>
       <c r="AD14" t="n">
-        <v>67</v>
+        <v>45</v>
       </c>
       <c r="AE14" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="AF14" t="n">
-        <v>450</v>
+        <v>550</v>
       </c>
       <c r="AG14" t="n">
         <v>2</v>
       </c>
       <c r="AH14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AI14" t="n">
         <v>3</v>
@@ -3057,12 +3060,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AO14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fio 1 e 2 Fios de espessura fina e comprimento curto.
-</t>
-        </is>
-      </c>
+      <c r="AO14" t="inlineStr"/>
       <c r="AP14" t="inlineStr"/>
       <c r="AQ14" t="inlineStr">
         <is>
@@ -3099,6 +3097,368 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-03-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>13/03/2025</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Darcilio Maester Neto</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Dr. Daniel</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Ana, angelica  (extra), larissa (extra)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>8</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3700</v>
+      </c>
+      <c r="J15" t="n">
+        <v>3700</v>
+      </c>
+      <c r="K15" t="n">
+        <v>127</v>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="Q15" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="R15" t="n">
+        <v>7</v>
+      </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="n">
+        <v>1</v>
+      </c>
+      <c r="U15" t="n">
+        <v>52</v>
+      </c>
+      <c r="V15" t="n">
+        <v>600</v>
+      </c>
+      <c r="W15" t="n">
+        <v>563</v>
+      </c>
+      <c r="X15" t="n">
+        <v>76</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>1300</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>1200</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>81</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>1400</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>42</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>550</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>537</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>3</v>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>nega</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fio 1 e 2 Fios de espessura grosso e comprimento longo.
+</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">angelica </t>
+        </is>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>larissa</t>
+        </is>
+      </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT15" t="inlineStr"/>
+      <c r="AU15" t="inlineStr"/>
+      <c r="AV15" t="inlineStr"/>
+      <c r="AW15" t="inlineStr"/>
+      <c r="AX15" t="inlineStr"/>
+      <c r="AY15" t="inlineStr"/>
+      <c r="AZ15" t="inlineStr"/>
+      <c r="BA15" t="inlineStr"/>
+      <c r="BB15" t="inlineStr"/>
+      <c r="BC15" t="inlineStr"/>
+      <c r="BD15" t="inlineStr"/>
+      <c r="BE15" t="inlineStr"/>
+      <c r="BF15" t="inlineStr"/>
+      <c r="BG15" t="inlineStr"/>
+      <c r="BH15" t="inlineStr">
+        <is>
+          <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-03-17</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>16/03/2025</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Thiago Domingos Chicarelli</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Dr. Arthur</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Aline, Natália, Ana</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>3</v>
+      </c>
+      <c r="I16" t="n">
+        <v>2513</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2253</v>
+      </c>
+      <c r="K16" t="n">
+        <v>52</v>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>130</v>
+      </c>
+      <c r="O16" t="n">
+        <v>130</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="R16" t="n">
+        <v>4</v>
+      </c>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="n">
+        <v>1</v>
+      </c>
+      <c r="U16" t="n">
+        <v>58</v>
+      </c>
+      <c r="V16" t="n">
+        <v>470</v>
+      </c>
+      <c r="W16" t="n">
+        <v>435</v>
+      </c>
+      <c r="X16" t="n">
+        <v>71</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>1070</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>1022</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>68</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>580</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>482</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>52</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>660</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>580</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>nega</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fio 1 e 2 Fios de espessura média e comprimento médio.
+</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr"/>
+      <c r="AR16" t="inlineStr"/>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr"/>
+      <c r="AU16" t="inlineStr"/>
+      <c r="AV16" t="inlineStr"/>
+      <c r="AW16" t="inlineStr"/>
+      <c r="AX16" t="inlineStr"/>
+      <c r="AY16" t="inlineStr"/>
+      <c r="AZ16" t="inlineStr"/>
+      <c r="BA16" t="inlineStr"/>
+      <c r="BB16" t="inlineStr"/>
+      <c r="BC16" t="inlineStr"/>
+      <c r="BD16" t="inlineStr"/>
+      <c r="BE16" t="inlineStr"/>
+      <c r="BF16" t="inlineStr"/>
+      <c r="BG16" t="inlineStr"/>
+      <c r="BH16" t="inlineStr">
+        <is>
+          <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Fix: Corrected duplicate patient entries in cirurgias.xlsx; data backed up.
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -1262,17 +1262,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-03-13</t>
+          <t>2025-03-07</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>12/03/2025</t>
+          <t>06/03/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Eduardo Roncaglia de Carvalho</t>
+          <t xml:space="preserve">Maurício Ronaldo Ribeiro </t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1282,37 +1282,33 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Dr. Daniel</t>
+          <t>Dr. Arthur</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Aline, Natália, thamara (extra)</t>
+          <t>Ana, angelica  (extra), larissa (extra)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="I5" t="n">
-        <v>3655</v>
+        <v>3737</v>
       </c>
       <c r="J5" t="n">
-        <v>2610</v>
+        <v>3737</v>
       </c>
       <c r="K5" t="n">
-        <v>105</v>
-      </c>
-      <c r="L5" t="n">
-        <v>840</v>
-      </c>
-      <c r="M5" t="n">
-        <v>200</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
@@ -1324,59 +1320,57 @@
         <v>0.85</v>
       </c>
       <c r="R5" t="n">
-        <v>4</v>
-      </c>
-      <c r="S5" t="n">
-        <v>5</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="S5" t="inlineStr"/>
       <c r="T5" t="n">
         <v>1</v>
       </c>
       <c r="U5" t="n">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="V5" t="n">
         <v>630</v>
       </c>
       <c r="W5" t="n">
-        <v>585</v>
+        <v>600</v>
       </c>
       <c r="X5" t="n">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="Y5" t="n">
-        <v>1300</v>
+        <v>1470</v>
       </c>
       <c r="Z5" t="n">
-        <v>1249</v>
+        <v>1400</v>
       </c>
       <c r="AA5" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="AB5" t="n">
-        <v>1300</v>
+        <v>1470</v>
       </c>
       <c r="AC5" t="n">
-        <v>1217</v>
+        <v>1400</v>
       </c>
       <c r="AD5" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="AE5" t="n">
-        <v>670</v>
+        <v>420</v>
       </c>
       <c r="AF5" t="n">
-        <v>604</v>
+        <v>387</v>
       </c>
       <c r="AG5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI5" t="n">
         <v>2</v>
       </c>
-      <c r="AI5" t="n">
-        <v>1</v>
-      </c>
       <c r="AJ5" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1402,23 +1396,22 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AO5" t="inlineStr">
-        <is>
-          <t>nega</t>
-        </is>
-      </c>
+      <c r="AO5" t="inlineStr"/>
       <c r="AP5" t="inlineStr">
         <is>
-          <t xml:space="preserve">fio 2  e 3 . Fios grossos  e médio . 
-</t>
+          <t xml:space="preserve"> fio 1 e 2 Fios fino e longo.</t>
         </is>
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>thamara</t>
-        </is>
-      </c>
-      <c r="AR5" t="inlineStr"/>
+          <t xml:space="preserve">angelica </t>
+        </is>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>larissa</t>
+        </is>
+      </c>
       <c r="AS5" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1629,17 +1622,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-03-07</t>
+          <t>2025-03-11</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06/03/2025</t>
+          <t>10/03/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maurício Ronaldo Ribeiro </t>
+          <t>José Antônio Tonetto Neto</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1649,7 +1642,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Dr. Arthur</t>
+          <t>Dr. Daniel</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1666,16 +1659,20 @@
         <v>6.5</v>
       </c>
       <c r="I7" t="n">
-        <v>3737</v>
+        <v>3498</v>
       </c>
       <c r="J7" t="n">
-        <v>3737</v>
+        <v>808</v>
       </c>
       <c r="K7" t="n">
-        <v>80</v>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+        <v>33</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1190</v>
+      </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
@@ -1684,63 +1681,65 @@
         </is>
       </c>
       <c r="Q7" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="R7" t="n">
+        <v>2</v>
+      </c>
+      <c r="S7" t="n">
         <v>7</v>
       </c>
-      <c r="S7" t="inlineStr"/>
       <c r="T7" t="n">
         <v>1</v>
       </c>
       <c r="U7" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="V7" t="n">
-        <v>630</v>
+        <v>700</v>
       </c>
       <c r="W7" t="n">
-        <v>600</v>
+        <v>668</v>
       </c>
       <c r="X7" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="Y7" t="n">
-        <v>1470</v>
+        <v>1050</v>
       </c>
       <c r="Z7" t="n">
-        <v>1400</v>
+        <v>930</v>
       </c>
       <c r="AA7" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="AB7" t="n">
-        <v>1470</v>
+        <v>1300</v>
       </c>
       <c r="AC7" t="n">
-        <v>1400</v>
+        <v>1200</v>
       </c>
       <c r="AD7" t="n">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="AE7" t="n">
-        <v>420</v>
+        <v>750</v>
       </c>
       <c r="AF7" t="n">
-        <v>387</v>
+        <v>700</v>
       </c>
       <c r="AG7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH7" t="n">
         <v>2</v>
-      </c>
-      <c r="AH7" t="n">
-        <v>3</v>
       </c>
       <c r="AI7" t="n">
         <v>2</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="AK7" t="inlineStr">
@@ -1763,10 +1762,15 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AO7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>nega</t>
+        </is>
+      </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> fio 1 e 2 Fios fino e longo.</t>
+          <t xml:space="preserve">fio 1 e 2 Fios fino e longo.
+</t>
         </is>
       </c>
       <c r="AQ7" t="inlineStr">
@@ -1817,7 +1821,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>José Antônio Tonetto Neto</t>
+          <t xml:space="preserve">Douglas Rodrigues Costa </t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1837,26 +1841,26 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="H8" t="n">
         <v>6.5</v>
       </c>
       <c r="I8" t="n">
-        <v>3498</v>
+        <v>4000</v>
       </c>
       <c r="J8" t="n">
-        <v>808</v>
+        <v>2710</v>
       </c>
       <c r="K8" t="n">
-        <v>33</v>
+        <v>99</v>
       </c>
       <c r="L8" t="n">
-        <v>1500</v>
+        <v>773</v>
       </c>
       <c r="M8" t="n">
-        <v>1190</v>
+        <v>517</v>
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
@@ -1869,7 +1873,7 @@
         <v>0.95</v>
       </c>
       <c r="R8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="S8" t="n">
         <v>7</v>
@@ -1878,60 +1882,60 @@
         <v>1</v>
       </c>
       <c r="U8" t="n">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="V8" t="n">
-        <v>700</v>
+        <v>450</v>
       </c>
       <c r="W8" t="n">
-        <v>668</v>
+        <v>360</v>
       </c>
       <c r="X8" t="n">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="Y8" t="n">
-        <v>1050</v>
+        <v>1700</v>
       </c>
       <c r="Z8" t="n">
-        <v>930</v>
+        <v>1590</v>
       </c>
       <c r="AA8" t="n">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="AB8" t="n">
-        <v>1300</v>
+        <v>1650</v>
       </c>
       <c r="AC8" t="n">
-        <v>1200</v>
+        <v>1544</v>
       </c>
       <c r="AD8" t="n">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="AE8" t="n">
-        <v>750</v>
+        <v>600</v>
       </c>
       <c r="AF8" t="n">
-        <v>700</v>
+        <v>503</v>
       </c>
       <c r="AG8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH8" t="n">
         <v>2</v>
       </c>
       <c r="AI8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="AK8" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
       <c r="AL8" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1952,12 +1956,7 @@
           <t>nega</t>
         </is>
       </c>
-      <c r="AP8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fio 1 e 2 Fios fino e longo.
-</t>
-        </is>
-      </c>
+      <c r="AP8" t="inlineStr"/>
       <c r="AQ8" t="inlineStr">
         <is>
           <t xml:space="preserve">angelica </t>
@@ -1996,17 +1995,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-03-11</t>
+          <t>2025-03-12</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>10/03/2025</t>
+          <t>11/03/2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Douglas Rodrigues Costa </t>
+          <t xml:space="preserve">Pedro Rafael de Almeida Picaccio </t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2030,77 +2029,75 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="I9" t="n">
-        <v>4000</v>
+        <v>4222</v>
       </c>
       <c r="J9" t="n">
-        <v>2710</v>
+        <v>3872</v>
       </c>
       <c r="K9" t="n">
-        <v>99</v>
-      </c>
-      <c r="L9" t="n">
-        <v>773</v>
-      </c>
-      <c r="M9" t="n">
-        <v>517</v>
-      </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+        <v>108</v>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="n">
+        <v>180</v>
+      </c>
+      <c r="O9" t="n">
+        <v>170</v>
+      </c>
       <c r="P9" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
       <c r="Q9" t="n">
-        <v>0.95</v>
+        <v>0.85</v>
       </c>
       <c r="R9" t="n">
-        <v>6</v>
-      </c>
-      <c r="S9" t="n">
-        <v>7</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="n">
         <v>1</v>
       </c>
       <c r="U9" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="V9" t="n">
-        <v>450</v>
+        <v>700</v>
       </c>
       <c r="W9" t="n">
-        <v>360</v>
+        <v>647</v>
       </c>
       <c r="X9" t="n">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="Y9" t="n">
-        <v>1700</v>
+        <v>1640</v>
       </c>
       <c r="Z9" t="n">
-        <v>1590</v>
+        <v>1575</v>
       </c>
       <c r="AA9" t="n">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="AB9" t="n">
         <v>1650</v>
       </c>
       <c r="AC9" t="n">
-        <v>1544</v>
+        <v>1600</v>
       </c>
       <c r="AD9" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="AE9" t="n">
-        <v>600</v>
+        <v>459</v>
       </c>
       <c r="AF9" t="n">
-        <v>503</v>
+        <v>400</v>
       </c>
       <c r="AG9" t="n">
         <v>2</v>
@@ -2123,7 +2120,7 @@
       </c>
       <c r="AL9" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="AM9" t="inlineStr">
@@ -2141,7 +2138,11 @@
           <t>nega</t>
         </is>
       </c>
-      <c r="AP9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>io 1 e 2 Fios finos e curtos</t>
+        </is>
+      </c>
       <c r="AQ9" t="inlineStr">
         <is>
           <t xml:space="preserve">angelica </t>
@@ -2190,7 +2191,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pedro Rafael de Almeida Picaccio </t>
+          <t xml:space="preserve">Rodolfo Carola </t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2200,7 +2201,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Dr. Daniel</t>
+          <t>Dr. Arthur</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -2210,79 +2211,79 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="I10" t="n">
-        <v>4222</v>
+        <v>3630</v>
       </c>
       <c r="J10" t="n">
-        <v>3872</v>
+        <v>3464</v>
       </c>
       <c r="K10" t="n">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
-        <v>180</v>
+        <v>85</v>
       </c>
       <c r="O10" t="n">
-        <v>170</v>
+        <v>81</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="Q10" t="n">
         <v>0.85</v>
       </c>
       <c r="R10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="n">
         <v>1</v>
       </c>
       <c r="U10" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="V10" t="n">
-        <v>700</v>
+        <v>500</v>
       </c>
       <c r="W10" t="n">
-        <v>647</v>
+        <v>433</v>
       </c>
       <c r="X10" t="n">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="Y10" t="n">
-        <v>1640</v>
+        <v>1550</v>
       </c>
       <c r="Z10" t="n">
-        <v>1575</v>
+        <v>1450</v>
       </c>
       <c r="AA10" t="n">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="AB10" t="n">
-        <v>1650</v>
+        <v>1300</v>
       </c>
       <c r="AC10" t="n">
-        <v>1600</v>
+        <v>1210</v>
       </c>
       <c r="AD10" t="n">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="AE10" t="n">
-        <v>459</v>
+        <v>600</v>
       </c>
       <c r="AF10" t="n">
-        <v>400</v>
+        <v>537</v>
       </c>
       <c r="AG10" t="n">
         <v>2</v>
@@ -2291,7 +2292,7 @@
         <v>2</v>
       </c>
       <c r="AI10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
@@ -2300,14 +2301,14 @@
       </c>
       <c r="AK10" t="inlineStr">
         <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="AL10" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
       <c r="AM10" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2325,7 +2326,7 @@
       </c>
       <c r="AP10" t="inlineStr">
         <is>
-          <t>io 1 e 2 Fios finos e curtos</t>
+          <t>fio 1 e 2 Fios de espessura média e comprimento médio</t>
         </is>
       </c>
       <c r="AQ10" t="inlineStr">
@@ -2366,17 +2367,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025-03-12</t>
+          <t>2025-03-13</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11/03/2025</t>
+          <t>12/03/2025</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rodolfo Carola </t>
+          <t>Eduardo Roncaglia de Carvalho</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2386,98 +2387,100 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Dr. Arthur</t>
+          <t>Dr. Daniel</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Ana, angelica  (extra), larissa (extra)</t>
+          <t>Aline, Natália, thamara (extra)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>6.5</v>
+        <v>5</v>
       </c>
       <c r="I11" t="n">
-        <v>3630</v>
+        <v>3655</v>
       </c>
       <c r="J11" t="n">
-        <v>3464</v>
+        <v>2610</v>
       </c>
       <c r="K11" t="n">
-        <v>123</v>
-      </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="n">
-        <v>85</v>
-      </c>
-      <c r="O11" t="n">
-        <v>81</v>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="L11" t="n">
+        <v>840</v>
+      </c>
+      <c r="M11" t="n">
+        <v>200</v>
+      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="Q11" t="n">
         <v>0.85</v>
       </c>
       <c r="R11" t="n">
+        <v>4</v>
+      </c>
+      <c r="S11" t="n">
         <v>5</v>
       </c>
-      <c r="S11" t="inlineStr"/>
       <c r="T11" t="n">
         <v>1</v>
       </c>
       <c r="U11" t="n">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="V11" t="n">
-        <v>500</v>
+        <v>630</v>
       </c>
       <c r="W11" t="n">
-        <v>433</v>
+        <v>585</v>
       </c>
       <c r="X11" t="n">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="Y11" t="n">
-        <v>1550</v>
+        <v>1300</v>
       </c>
       <c r="Z11" t="n">
-        <v>1450</v>
+        <v>1249</v>
       </c>
       <c r="AA11" t="n">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="AB11" t="n">
         <v>1300</v>
       </c>
       <c r="AC11" t="n">
-        <v>1210</v>
+        <v>1217</v>
       </c>
       <c r="AD11" t="n">
-        <v>68</v>
+        <v>48</v>
       </c>
       <c r="AE11" t="n">
-        <v>600</v>
+        <v>670</v>
       </c>
       <c r="AF11" t="n">
-        <v>537</v>
+        <v>604</v>
       </c>
       <c r="AG11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH11" t="n">
         <v>2</v>
       </c>
       <c r="AI11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
@@ -2491,7 +2494,7 @@
       </c>
       <c r="AL11" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="AM11" t="inlineStr">
@@ -2511,19 +2514,16 @@
       </c>
       <c r="AP11" t="inlineStr">
         <is>
-          <t>fio 1 e 2 Fios de espessura média e comprimento médio</t>
+          <t xml:space="preserve">fio 2  e 3 . Fios grossos  e médio . 
+</t>
         </is>
       </c>
       <c r="AQ11" t="inlineStr">
         <is>
-          <t xml:space="preserve">angelica </t>
-        </is>
-      </c>
-      <c r="AR11" t="inlineStr">
-        <is>
-          <t>larissa</t>
-        </is>
-      </c>
+          <t>thamara</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="inlineStr">
         <is>
           <t>Não</t>

</xml_diff>

<commit_message>
Improve data handling and error management in surgery data saving.  Added more robust date handling and updated field mappings for improved data consistency.
Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 164eb805-1c2b-4cd9-a960-65b2f31dbc5f
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/8c7417ff-25e3-4894-9a88-ca4d88413804/02021399-9e25-4909-a960-a62ccbcbf5ba.jpg
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH16"/>
+  <dimension ref="A1:BV17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -727,6 +727,76 @@
       <c r="BH1" s="1" t="inlineStr">
         <is>
           <t>bloqueio_data</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>Data (DD/MM/AAAA)</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>Paciente</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>Médico</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>Hora da Cirurgia (HH:MM)</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>Tempo de Cirurgia (horas)</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>Total de Folículos</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>Frente</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>Densidade Scketh</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>Coroa</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>Scalpe</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>Península Direita</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>Península Esquerda</t>
         </is>
       </c>
     </row>
@@ -897,6 +967,20 @@
           <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
         </is>
       </c>
+      <c r="BI2" t="inlineStr"/>
+      <c r="BJ2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="inlineStr"/>
+      <c r="BM2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr"/>
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
+      <c r="BU2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1075,6 +1159,20 @@
           <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
         </is>
       </c>
+      <c r="BI3" t="inlineStr"/>
+      <c r="BJ3" t="inlineStr"/>
+      <c r="BK3" t="inlineStr"/>
+      <c r="BL3" t="inlineStr"/>
+      <c r="BM3" t="inlineStr"/>
+      <c r="BN3" t="inlineStr"/>
+      <c r="BO3" t="inlineStr"/>
+      <c r="BP3" t="inlineStr"/>
+      <c r="BQ3" t="inlineStr"/>
+      <c r="BR3" t="inlineStr"/>
+      <c r="BS3" t="inlineStr"/>
+      <c r="BT3" t="inlineStr"/>
+      <c r="BU3" t="inlineStr"/>
+      <c r="BV3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1258,6 +1356,20 @@
           <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
         </is>
       </c>
+      <c r="BI4" t="inlineStr"/>
+      <c r="BJ4" t="inlineStr"/>
+      <c r="BK4" t="inlineStr"/>
+      <c r="BL4" t="inlineStr"/>
+      <c r="BM4" t="inlineStr"/>
+      <c r="BN4" t="inlineStr"/>
+      <c r="BO4" t="inlineStr"/>
+      <c r="BP4" t="inlineStr"/>
+      <c r="BQ4" t="inlineStr"/>
+      <c r="BR4" t="inlineStr"/>
+      <c r="BS4" t="inlineStr"/>
+      <c r="BT4" t="inlineStr"/>
+      <c r="BU4" t="inlineStr"/>
+      <c r="BV4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1436,6 +1548,20 @@
           <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
         </is>
       </c>
+      <c r="BI5" t="inlineStr"/>
+      <c r="BJ5" t="inlineStr"/>
+      <c r="BK5" t="inlineStr"/>
+      <c r="BL5" t="inlineStr"/>
+      <c r="BM5" t="inlineStr"/>
+      <c r="BN5" t="inlineStr"/>
+      <c r="BO5" t="inlineStr"/>
+      <c r="BP5" t="inlineStr"/>
+      <c r="BQ5" t="inlineStr"/>
+      <c r="BR5" t="inlineStr"/>
+      <c r="BS5" t="inlineStr"/>
+      <c r="BT5" t="inlineStr"/>
+      <c r="BU5" t="inlineStr"/>
+      <c r="BV5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1618,6 +1744,20 @@
           <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
         </is>
       </c>
+      <c r="BI6" t="inlineStr"/>
+      <c r="BJ6" t="inlineStr"/>
+      <c r="BK6" t="inlineStr"/>
+      <c r="BL6" t="inlineStr"/>
+      <c r="BM6" t="inlineStr"/>
+      <c r="BN6" t="inlineStr"/>
+      <c r="BO6" t="inlineStr"/>
+      <c r="BP6" t="inlineStr"/>
+      <c r="BQ6" t="inlineStr"/>
+      <c r="BR6" t="inlineStr"/>
+      <c r="BS6" t="inlineStr"/>
+      <c r="BT6" t="inlineStr"/>
+      <c r="BU6" t="inlineStr"/>
+      <c r="BV6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1807,6 +1947,20 @@
           <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
         </is>
       </c>
+      <c r="BI7" t="inlineStr"/>
+      <c r="BJ7" t="inlineStr"/>
+      <c r="BK7" t="inlineStr"/>
+      <c r="BL7" t="inlineStr"/>
+      <c r="BM7" t="inlineStr"/>
+      <c r="BN7" t="inlineStr"/>
+      <c r="BO7" t="inlineStr"/>
+      <c r="BP7" t="inlineStr"/>
+      <c r="BQ7" t="inlineStr"/>
+      <c r="BR7" t="inlineStr"/>
+      <c r="BS7" t="inlineStr"/>
+      <c r="BT7" t="inlineStr"/>
+      <c r="BU7" t="inlineStr"/>
+      <c r="BV7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1991,6 +2145,20 @@
           <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
         </is>
       </c>
+      <c r="BI8" t="inlineStr"/>
+      <c r="BJ8" t="inlineStr"/>
+      <c r="BK8" t="inlineStr"/>
+      <c r="BL8" t="inlineStr"/>
+      <c r="BM8" t="inlineStr"/>
+      <c r="BN8" t="inlineStr"/>
+      <c r="BO8" t="inlineStr"/>
+      <c r="BP8" t="inlineStr"/>
+      <c r="BQ8" t="inlineStr"/>
+      <c r="BR8" t="inlineStr"/>
+      <c r="BS8" t="inlineStr"/>
+      <c r="BT8" t="inlineStr"/>
+      <c r="BU8" t="inlineStr"/>
+      <c r="BV8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2177,6 +2345,20 @@
           <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
         </is>
       </c>
+      <c r="BI9" t="inlineStr"/>
+      <c r="BJ9" t="inlineStr"/>
+      <c r="BK9" t="inlineStr"/>
+      <c r="BL9" t="inlineStr"/>
+      <c r="BM9" t="inlineStr"/>
+      <c r="BN9" t="inlineStr"/>
+      <c r="BO9" t="inlineStr"/>
+      <c r="BP9" t="inlineStr"/>
+      <c r="BQ9" t="inlineStr"/>
+      <c r="BR9" t="inlineStr"/>
+      <c r="BS9" t="inlineStr"/>
+      <c r="BT9" t="inlineStr"/>
+      <c r="BU9" t="inlineStr"/>
+      <c r="BV9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2363,6 +2545,20 @@
           <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
         </is>
       </c>
+      <c r="BI10" t="inlineStr"/>
+      <c r="BJ10" t="inlineStr"/>
+      <c r="BK10" t="inlineStr"/>
+      <c r="BL10" t="inlineStr"/>
+      <c r="BM10" t="inlineStr"/>
+      <c r="BN10" t="inlineStr"/>
+      <c r="BO10" t="inlineStr"/>
+      <c r="BP10" t="inlineStr"/>
+      <c r="BQ10" t="inlineStr"/>
+      <c r="BR10" t="inlineStr"/>
+      <c r="BS10" t="inlineStr"/>
+      <c r="BT10" t="inlineStr"/>
+      <c r="BU10" t="inlineStr"/>
+      <c r="BV10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2548,6 +2744,20 @@
           <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
         </is>
       </c>
+      <c r="BI11" t="inlineStr"/>
+      <c r="BJ11" t="inlineStr"/>
+      <c r="BK11" t="inlineStr"/>
+      <c r="BL11" t="inlineStr"/>
+      <c r="BM11" t="inlineStr"/>
+      <c r="BN11" t="inlineStr"/>
+      <c r="BO11" t="inlineStr"/>
+      <c r="BP11" t="inlineStr"/>
+      <c r="BQ11" t="inlineStr"/>
+      <c r="BR11" t="inlineStr"/>
+      <c r="BS11" t="inlineStr"/>
+      <c r="BT11" t="inlineStr"/>
+      <c r="BU11" t="inlineStr"/>
+      <c r="BV11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2737,6 +2947,20 @@
           <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
         </is>
       </c>
+      <c r="BI12" t="inlineStr"/>
+      <c r="BJ12" t="inlineStr"/>
+      <c r="BK12" t="inlineStr"/>
+      <c r="BL12" t="inlineStr"/>
+      <c r="BM12" t="inlineStr"/>
+      <c r="BN12" t="inlineStr"/>
+      <c r="BO12" t="inlineStr"/>
+      <c r="BP12" t="inlineStr"/>
+      <c r="BQ12" t="inlineStr"/>
+      <c r="BR12" t="inlineStr"/>
+      <c r="BS12" t="inlineStr"/>
+      <c r="BT12" t="inlineStr"/>
+      <c r="BU12" t="inlineStr"/>
+      <c r="BV12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2922,6 +3146,20 @@
           <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
         </is>
       </c>
+      <c r="BI13" t="inlineStr"/>
+      <c r="BJ13" t="inlineStr"/>
+      <c r="BK13" t="inlineStr"/>
+      <c r="BL13" t="inlineStr"/>
+      <c r="BM13" t="inlineStr"/>
+      <c r="BN13" t="inlineStr"/>
+      <c r="BO13" t="inlineStr"/>
+      <c r="BP13" t="inlineStr"/>
+      <c r="BQ13" t="inlineStr"/>
+      <c r="BR13" t="inlineStr"/>
+      <c r="BS13" t="inlineStr"/>
+      <c r="BT13" t="inlineStr"/>
+      <c r="BU13" t="inlineStr"/>
+      <c r="BV13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3096,6 +3334,20 @@
           <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
         </is>
       </c>
+      <c r="BI14" t="inlineStr"/>
+      <c r="BJ14" t="inlineStr"/>
+      <c r="BK14" t="inlineStr"/>
+      <c r="BL14" t="inlineStr"/>
+      <c r="BM14" t="inlineStr"/>
+      <c r="BN14" t="inlineStr"/>
+      <c r="BO14" t="inlineStr"/>
+      <c r="BP14" t="inlineStr"/>
+      <c r="BQ14" t="inlineStr"/>
+      <c r="BR14" t="inlineStr"/>
+      <c r="BS14" t="inlineStr"/>
+      <c r="BT14" t="inlineStr"/>
+      <c r="BU14" t="inlineStr"/>
+      <c r="BV14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3279,6 +3531,20 @@
           <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
         </is>
       </c>
+      <c r="BI15" t="inlineStr"/>
+      <c r="BJ15" t="inlineStr"/>
+      <c r="BK15" t="inlineStr"/>
+      <c r="BL15" t="inlineStr"/>
+      <c r="BM15" t="inlineStr"/>
+      <c r="BN15" t="inlineStr"/>
+      <c r="BO15" t="inlineStr"/>
+      <c r="BP15" t="inlineStr"/>
+      <c r="BQ15" t="inlineStr"/>
+      <c r="BR15" t="inlineStr"/>
+      <c r="BS15" t="inlineStr"/>
+      <c r="BT15" t="inlineStr"/>
+      <c r="BU15" t="inlineStr"/>
+      <c r="BV15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3458,6 +3724,152 @@
           <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
         </is>
       </c>
+      <c r="BI16" t="inlineStr"/>
+      <c r="BJ16" t="inlineStr"/>
+      <c r="BK16" t="inlineStr"/>
+      <c r="BL16" t="inlineStr"/>
+      <c r="BM16" t="inlineStr"/>
+      <c r="BN16" t="inlineStr"/>
+      <c r="BO16" t="inlineStr"/>
+      <c r="BP16" t="inlineStr"/>
+      <c r="BQ16" t="inlineStr"/>
+      <c r="BR16" t="inlineStr"/>
+      <c r="BS16" t="inlineStr"/>
+      <c r="BT16" t="inlineStr"/>
+      <c r="BU16" t="inlineStr"/>
+      <c r="BV16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr"/>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
+      <c r="AG17" t="inlineStr"/>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr"/>
+      <c r="AM17" t="inlineStr"/>
+      <c r="AN17" t="inlineStr"/>
+      <c r="AO17" t="inlineStr"/>
+      <c r="AP17" t="inlineStr"/>
+      <c r="AQ17" t="inlineStr"/>
+      <c r="AR17" t="inlineStr"/>
+      <c r="AS17" t="inlineStr"/>
+      <c r="AT17" t="inlineStr"/>
+      <c r="AU17" t="inlineStr"/>
+      <c r="AV17" t="inlineStr"/>
+      <c r="AW17" t="inlineStr"/>
+      <c r="AX17" t="inlineStr"/>
+      <c r="AY17" t="inlineStr"/>
+      <c r="AZ17" t="inlineStr"/>
+      <c r="BA17" t="inlineStr"/>
+      <c r="BB17" t="inlineStr"/>
+      <c r="BC17" t="inlineStr"/>
+      <c r="BD17" t="inlineStr"/>
+      <c r="BE17" t="inlineStr"/>
+      <c r="BF17" t="inlineStr"/>
+      <c r="BG17" t="inlineStr"/>
+      <c r="BH17" t="inlineStr"/>
+      <c r="BI17" t="inlineStr">
+        <is>
+          <t>07/04/2025</t>
+        </is>
+      </c>
+      <c r="BJ17" t="inlineStr">
+        <is>
+          <t>Teste</t>
+        </is>
+      </c>
+      <c r="BK17" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="BL17" t="inlineStr">
+        <is>
+          <t>Dr. Silva</t>
+        </is>
+      </c>
+      <c r="BM17" t="inlineStr">
+        <is>
+          <t>Equipe 1</t>
+        </is>
+      </c>
+      <c r="BN17" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="BO17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="BP17" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="BQ17" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="BR17" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="BS17" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="BT17" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="BU17" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="BV17" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add missing button to patient registration form
Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 164eb805-1c2b-4cd9-a960-65b2f31dbc5f
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/8c7417ff-25e3-4894-9a88-ca4d88413804/3ce59808-6c3f-41a6-b8be-7d98152ffa80.jpg
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BV17"/>
+  <dimension ref="A1:BV18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3830,46 +3830,234 @@
           <t>10:00</t>
         </is>
       </c>
-      <c r="BO17" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="BP17" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="BQ17" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="BR17" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
-      <c r="BS17" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="BT17" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="BU17" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="BV17" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="BO17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BP17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="BQ17" t="n">
+        <v>500</v>
+      </c>
+      <c r="BR17" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="BS17" t="n">
+        <v>300</v>
+      </c>
+      <c r="BT17" t="n">
+        <v>100</v>
+      </c>
+      <c r="BU17" t="n">
+        <v>50</v>
+      </c>
+      <c r="BV17" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-04-26</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>teste1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Dra. Natalia</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Thamara Maciel</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AL18" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO18" t="inlineStr"/>
+      <c r="AP18" t="inlineStr"/>
+      <c r="AQ18" t="inlineStr"/>
+      <c r="AR18" t="inlineStr"/>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT18" t="inlineStr"/>
+      <c r="AU18" t="inlineStr"/>
+      <c r="AV18" t="inlineStr"/>
+      <c r="AW18" t="inlineStr"/>
+      <c r="AX18" t="inlineStr"/>
+      <c r="AY18" t="inlineStr"/>
+      <c r="AZ18" t="inlineStr"/>
+      <c r="BA18" t="inlineStr"/>
+      <c r="BB18" t="inlineStr"/>
+      <c r="BC18" t="inlineStr"/>
+      <c r="BD18" t="inlineStr"/>
+      <c r="BE18" t="inlineStr"/>
+      <c r="BF18" t="inlineStr"/>
+      <c r="BG18" t="inlineStr"/>
+      <c r="BH18" t="inlineStr"/>
+      <c r="BI18" t="inlineStr"/>
+      <c r="BJ18" t="inlineStr"/>
+      <c r="BK18" t="inlineStr"/>
+      <c r="BL18" t="inlineStr"/>
+      <c r="BM18" t="inlineStr"/>
+      <c r="BN18" t="inlineStr"/>
+      <c r="BO18" t="inlineStr"/>
+      <c r="BP18" t="inlineStr"/>
+      <c r="BQ18" t="inlineStr"/>
+      <c r="BR18" t="inlineStr"/>
+      <c r="BS18" t="inlineStr"/>
+      <c r="BT18" t="inlineStr"/>
+      <c r="BU18" t="inlineStr"/>
+      <c r="BV18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Record changes to surgical procedures and create backups for safety
Back up the "cirurgias.xlsx" file and store it in the data_backup directory.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BV18"/>
+  <dimension ref="A1:BV19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3887,15 +3887,11 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="H18" t="n">
+        <v>5</v>
+      </c>
+      <c r="I18" t="n">
+        <v>6</v>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
@@ -3908,92 +3904,58 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="Q18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="R18" t="n">
+        <v>6</v>
       </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="X18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="Y18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="Z18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="AA18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="AB18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="AC18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="AD18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="AE18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="AF18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="AG18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AH18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AI18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="U18" t="n">
+        <v>6</v>
+      </c>
+      <c r="V18" t="n">
+        <v>6</v>
+      </c>
+      <c r="W18" t="n">
+        <v>6</v>
+      </c>
+      <c r="X18" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>1</v>
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
@@ -4059,6 +4021,218 @@
       <c r="BU18" t="inlineStr"/>
       <c r="BV18" t="inlineStr"/>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-06-12</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">arthur </t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Dra. Leticia</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Angélica Sousa</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>0,90x5mm</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AI19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN19" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO19" t="inlineStr"/>
+      <c r="AP19" t="inlineStr"/>
+      <c r="AQ19" t="inlineStr"/>
+      <c r="AR19" t="inlineStr"/>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT19" t="inlineStr"/>
+      <c r="AU19" t="inlineStr"/>
+      <c r="AV19" t="inlineStr"/>
+      <c r="AW19" t="inlineStr"/>
+      <c r="AX19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr"/>
+      <c r="AZ19" t="inlineStr"/>
+      <c r="BA19" t="inlineStr"/>
+      <c r="BB19" t="inlineStr"/>
+      <c r="BC19" t="inlineStr"/>
+      <c r="BD19" t="inlineStr"/>
+      <c r="BE19" t="inlineStr"/>
+      <c r="BF19" t="inlineStr"/>
+      <c r="BG19" t="inlineStr"/>
+      <c r="BH19" t="inlineStr"/>
+      <c r="BI19" t="inlineStr"/>
+      <c r="BJ19" t="inlineStr"/>
+      <c r="BK19" t="inlineStr"/>
+      <c r="BL19" t="inlineStr"/>
+      <c r="BM19" t="inlineStr"/>
+      <c r="BN19" t="inlineStr"/>
+      <c r="BO19" t="inlineStr"/>
+      <c r="BP19" t="inlineStr"/>
+      <c r="BQ19" t="inlineStr"/>
+      <c r="BR19" t="inlineStr"/>
+      <c r="BS19" t="inlineStr"/>
+      <c r="BT19" t="inlineStr"/>
+      <c r="BU19" t="inlineStr"/>
+      <c r="BV19" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record all intraoperative details and properly save the surgical team
Adds tracking for sedation and bleeding and fixes saving all team members to the database.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: c6555968-a064-4ba3-9362-39daf87f19d4
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/8c7417ff-25e3-4894-9a88-ca4d88413804/f41b7624-5334-434e-88a8-7ff2ac78a32c.jpg
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BV19"/>
+  <dimension ref="A1:CA20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -797,6 +797,31 @@
       <c r="BV1" s="1" t="inlineStr">
         <is>
           <t>Península Esquerda</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>body_hair_check</t>
+        </is>
+      </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>barba_check</t>
+        </is>
+      </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>peitoral_check</t>
+        </is>
+      </c>
+      <c r="BZ1" s="1" t="inlineStr">
+        <is>
+          <t>abdome_check</t>
+        </is>
+      </c>
+      <c r="CA1" s="1" t="inlineStr">
+        <is>
+          <t>dorso_check</t>
         </is>
       </c>
     </row>
@@ -981,6 +1006,11 @@
       <c r="BT2" t="inlineStr"/>
       <c r="BU2" t="inlineStr"/>
       <c r="BV2" t="inlineStr"/>
+      <c r="BW2" t="inlineStr"/>
+      <c r="BX2" t="inlineStr"/>
+      <c r="BY2" t="inlineStr"/>
+      <c r="BZ2" t="inlineStr"/>
+      <c r="CA2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1173,6 +1203,11 @@
       <c r="BT3" t="inlineStr"/>
       <c r="BU3" t="inlineStr"/>
       <c r="BV3" t="inlineStr"/>
+      <c r="BW3" t="inlineStr"/>
+      <c r="BX3" t="inlineStr"/>
+      <c r="BY3" t="inlineStr"/>
+      <c r="BZ3" t="inlineStr"/>
+      <c r="CA3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1370,6 +1405,11 @@
       <c r="BT4" t="inlineStr"/>
       <c r="BU4" t="inlineStr"/>
       <c r="BV4" t="inlineStr"/>
+      <c r="BW4" t="inlineStr"/>
+      <c r="BX4" t="inlineStr"/>
+      <c r="BY4" t="inlineStr"/>
+      <c r="BZ4" t="inlineStr"/>
+      <c r="CA4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1562,6 +1602,11 @@
       <c r="BT5" t="inlineStr"/>
       <c r="BU5" t="inlineStr"/>
       <c r="BV5" t="inlineStr"/>
+      <c r="BW5" t="inlineStr"/>
+      <c r="BX5" t="inlineStr"/>
+      <c r="BY5" t="inlineStr"/>
+      <c r="BZ5" t="inlineStr"/>
+      <c r="CA5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1758,6 +1803,11 @@
       <c r="BT6" t="inlineStr"/>
       <c r="BU6" t="inlineStr"/>
       <c r="BV6" t="inlineStr"/>
+      <c r="BW6" t="inlineStr"/>
+      <c r="BX6" t="inlineStr"/>
+      <c r="BY6" t="inlineStr"/>
+      <c r="BZ6" t="inlineStr"/>
+      <c r="CA6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1961,6 +2011,11 @@
       <c r="BT7" t="inlineStr"/>
       <c r="BU7" t="inlineStr"/>
       <c r="BV7" t="inlineStr"/>
+      <c r="BW7" t="inlineStr"/>
+      <c r="BX7" t="inlineStr"/>
+      <c r="BY7" t="inlineStr"/>
+      <c r="BZ7" t="inlineStr"/>
+      <c r="CA7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2159,6 +2214,11 @@
       <c r="BT8" t="inlineStr"/>
       <c r="BU8" t="inlineStr"/>
       <c r="BV8" t="inlineStr"/>
+      <c r="BW8" t="inlineStr"/>
+      <c r="BX8" t="inlineStr"/>
+      <c r="BY8" t="inlineStr"/>
+      <c r="BZ8" t="inlineStr"/>
+      <c r="CA8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2359,6 +2419,11 @@
       <c r="BT9" t="inlineStr"/>
       <c r="BU9" t="inlineStr"/>
       <c r="BV9" t="inlineStr"/>
+      <c r="BW9" t="inlineStr"/>
+      <c r="BX9" t="inlineStr"/>
+      <c r="BY9" t="inlineStr"/>
+      <c r="BZ9" t="inlineStr"/>
+      <c r="CA9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2559,6 +2624,11 @@
       <c r="BT10" t="inlineStr"/>
       <c r="BU10" t="inlineStr"/>
       <c r="BV10" t="inlineStr"/>
+      <c r="BW10" t="inlineStr"/>
+      <c r="BX10" t="inlineStr"/>
+      <c r="BY10" t="inlineStr"/>
+      <c r="BZ10" t="inlineStr"/>
+      <c r="CA10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2758,6 +2828,11 @@
       <c r="BT11" t="inlineStr"/>
       <c r="BU11" t="inlineStr"/>
       <c r="BV11" t="inlineStr"/>
+      <c r="BW11" t="inlineStr"/>
+      <c r="BX11" t="inlineStr"/>
+      <c r="BY11" t="inlineStr"/>
+      <c r="BZ11" t="inlineStr"/>
+      <c r="CA11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2961,6 +3036,11 @@
       <c r="BT12" t="inlineStr"/>
       <c r="BU12" t="inlineStr"/>
       <c r="BV12" t="inlineStr"/>
+      <c r="BW12" t="inlineStr"/>
+      <c r="BX12" t="inlineStr"/>
+      <c r="BY12" t="inlineStr"/>
+      <c r="BZ12" t="inlineStr"/>
+      <c r="CA12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3160,6 +3240,11 @@
       <c r="BT13" t="inlineStr"/>
       <c r="BU13" t="inlineStr"/>
       <c r="BV13" t="inlineStr"/>
+      <c r="BW13" t="inlineStr"/>
+      <c r="BX13" t="inlineStr"/>
+      <c r="BY13" t="inlineStr"/>
+      <c r="BZ13" t="inlineStr"/>
+      <c r="CA13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3348,6 +3433,11 @@
       <c r="BT14" t="inlineStr"/>
       <c r="BU14" t="inlineStr"/>
       <c r="BV14" t="inlineStr"/>
+      <c r="BW14" t="inlineStr"/>
+      <c r="BX14" t="inlineStr"/>
+      <c r="BY14" t="inlineStr"/>
+      <c r="BZ14" t="inlineStr"/>
+      <c r="CA14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3545,6 +3635,11 @@
       <c r="BT15" t="inlineStr"/>
       <c r="BU15" t="inlineStr"/>
       <c r="BV15" t="inlineStr"/>
+      <c r="BW15" t="inlineStr"/>
+      <c r="BX15" t="inlineStr"/>
+      <c r="BY15" t="inlineStr"/>
+      <c r="BZ15" t="inlineStr"/>
+      <c r="CA15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3738,6 +3833,11 @@
       <c r="BT16" t="inlineStr"/>
       <c r="BU16" t="inlineStr"/>
       <c r="BV16" t="inlineStr"/>
+      <c r="BW16" t="inlineStr"/>
+      <c r="BX16" t="inlineStr"/>
+      <c r="BY16" t="inlineStr"/>
+      <c r="BZ16" t="inlineStr"/>
+      <c r="CA16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
@@ -3854,6 +3954,11 @@
       <c r="BV17" t="n">
         <v>50</v>
       </c>
+      <c r="BW17" t="inlineStr"/>
+      <c r="BX17" t="inlineStr"/>
+      <c r="BY17" t="inlineStr"/>
+      <c r="BZ17" t="inlineStr"/>
+      <c r="CA17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4020,6 +4125,11 @@
       <c r="BT18" t="inlineStr"/>
       <c r="BU18" t="inlineStr"/>
       <c r="BV18" t="inlineStr"/>
+      <c r="BW18" t="inlineStr"/>
+      <c r="BX18" t="inlineStr"/>
+      <c r="BY18" t="inlineStr"/>
+      <c r="BZ18" t="inlineStr"/>
+      <c r="CA18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4053,25 +4163,17 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>3000</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="H19" t="n">
+        <v>5</v>
+      </c>
+      <c r="I19" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J19" t="n">
+        <v>100</v>
+      </c>
+      <c r="K19" t="n">
+        <v>10</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
@@ -4087,87 +4189,55 @@
           <t>0,90x5mm</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="R19" t="n">
+        <v>3</v>
       </c>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="Y19" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="Z19" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AA19" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AB19" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AC19" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AD19" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AE19" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AF19" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AG19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AH19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AI19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="U19" t="n">
+        <v>10</v>
+      </c>
+      <c r="V19" t="n">
+        <v>10</v>
+      </c>
+      <c r="W19" t="n">
+        <v>10</v>
+      </c>
+      <c r="X19" t="n">
+        <v>10</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>10</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>1</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
@@ -4232,6 +4302,300 @@
       <c r="BT19" t="inlineStr"/>
       <c r="BU19" t="inlineStr"/>
       <c r="BV19" t="inlineStr"/>
+      <c r="BW19" t="inlineStr"/>
+      <c r="BX19" t="inlineStr"/>
+      <c r="BY19" t="inlineStr"/>
+      <c r="BZ19" t="inlineStr"/>
+      <c r="CA19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-06-27</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Jonatas Luiz dos Santos</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Dr. Arthur</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Aline</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>4009</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>848</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>3161</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>199</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>0,90x4mm</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>550</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>387</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>725</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>840</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>695</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>530</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>372</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AI20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK20" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL20" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>nega</t>
+        </is>
+      </c>
+      <c r="AP20" t="inlineStr"/>
+      <c r="AQ20" t="inlineStr"/>
+      <c r="AR20" t="inlineStr"/>
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT20" t="inlineStr"/>
+      <c r="AU20" t="inlineStr"/>
+      <c r="AV20" t="inlineStr">
+        <is>
+          <t>800</t>
+        </is>
+      </c>
+      <c r="AW20" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="AX20" t="inlineStr"/>
+      <c r="AY20" t="inlineStr">
+        <is>
+          <t>1400</t>
+        </is>
+      </c>
+      <c r="AZ20" t="inlineStr">
+        <is>
+          <t>744</t>
+        </is>
+      </c>
+      <c r="BA20" t="inlineStr"/>
+      <c r="BB20" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="BC20" t="inlineStr">
+        <is>
+          <t>657</t>
+        </is>
+      </c>
+      <c r="BD20" t="inlineStr"/>
+      <c r="BE20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BF20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BG20" t="inlineStr"/>
+      <c r="BH20" t="inlineStr"/>
+      <c r="BI20" t="inlineStr"/>
+      <c r="BJ20" t="inlineStr"/>
+      <c r="BK20" t="inlineStr"/>
+      <c r="BL20" t="inlineStr"/>
+      <c r="BM20" t="inlineStr"/>
+      <c r="BN20" t="inlineStr"/>
+      <c r="BO20" t="inlineStr"/>
+      <c r="BP20" t="inlineStr"/>
+      <c r="BQ20" t="inlineStr"/>
+      <c r="BR20" t="inlineStr"/>
+      <c r="BS20" t="inlineStr"/>
+      <c r="BT20" t="inlineStr"/>
+      <c r="BU20" t="inlineStr"/>
+      <c r="BV20" t="inlineStr"/>
+      <c r="BW20" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="BX20" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="BY20" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="BZ20" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="CA20" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Create a backup of surgical data to ensure ongoing availability
Adds a surgical data backup to data_backup/cirurgias_20250611_193313.xlsx.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 7910296b-13ef-440a-bc5d-2363bc1496e5
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/8c7417ff-25e3-4894-9a88-ca4d88413804/0a89cb4b-6992-46e7-963b-bad66b6e3414.jpg
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CA20"/>
+  <dimension ref="A1:CH21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -822,6 +822,41 @@
       <c r="CA1" s="1" t="inlineStr">
         <is>
           <t>dorso_check</t>
+        </is>
+      </c>
+      <c r="CB1" s="1" t="inlineStr">
+        <is>
+          <t>Hora da Cirurgia</t>
+        </is>
+      </c>
+      <c r="CC1" s="1" t="inlineStr">
+        <is>
+          <t>Tempo de Cirurgia (h)</t>
+        </is>
+      </c>
+      <c r="CD1" s="1" t="inlineStr">
+        <is>
+          <t>Densidade Sketch</t>
+        </is>
+      </c>
+      <c r="CE1" s="1" t="inlineStr">
+        <is>
+          <t>pelos_corporais</t>
+        </is>
+      </c>
+      <c r="CF1" s="1" t="inlineStr">
+        <is>
+          <t>pernas_furos</t>
+        </is>
+      </c>
+      <c r="CG1" s="1" t="inlineStr">
+        <is>
+          <t>pernas_fios</t>
+        </is>
+      </c>
+      <c r="CH1" s="1" t="inlineStr">
+        <is>
+          <t>pernas_comentarios</t>
         </is>
       </c>
     </row>
@@ -1011,6 +1046,13 @@
       <c r="BY2" t="inlineStr"/>
       <c r="BZ2" t="inlineStr"/>
       <c r="CA2" t="inlineStr"/>
+      <c r="CB2" t="inlineStr"/>
+      <c r="CC2" t="inlineStr"/>
+      <c r="CD2" t="inlineStr"/>
+      <c r="CE2" t="inlineStr"/>
+      <c r="CF2" t="inlineStr"/>
+      <c r="CG2" t="inlineStr"/>
+      <c r="CH2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1208,6 +1250,13 @@
       <c r="BY3" t="inlineStr"/>
       <c r="BZ3" t="inlineStr"/>
       <c r="CA3" t="inlineStr"/>
+      <c r="CB3" t="inlineStr"/>
+      <c r="CC3" t="inlineStr"/>
+      <c r="CD3" t="inlineStr"/>
+      <c r="CE3" t="inlineStr"/>
+      <c r="CF3" t="inlineStr"/>
+      <c r="CG3" t="inlineStr"/>
+      <c r="CH3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1410,6 +1459,13 @@
       <c r="BY4" t="inlineStr"/>
       <c r="BZ4" t="inlineStr"/>
       <c r="CA4" t="inlineStr"/>
+      <c r="CB4" t="inlineStr"/>
+      <c r="CC4" t="inlineStr"/>
+      <c r="CD4" t="inlineStr"/>
+      <c r="CE4" t="inlineStr"/>
+      <c r="CF4" t="inlineStr"/>
+      <c r="CG4" t="inlineStr"/>
+      <c r="CH4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1607,6 +1663,13 @@
       <c r="BY5" t="inlineStr"/>
       <c r="BZ5" t="inlineStr"/>
       <c r="CA5" t="inlineStr"/>
+      <c r="CB5" t="inlineStr"/>
+      <c r="CC5" t="inlineStr"/>
+      <c r="CD5" t="inlineStr"/>
+      <c r="CE5" t="inlineStr"/>
+      <c r="CF5" t="inlineStr"/>
+      <c r="CG5" t="inlineStr"/>
+      <c r="CH5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1808,6 +1871,13 @@
       <c r="BY6" t="inlineStr"/>
       <c r="BZ6" t="inlineStr"/>
       <c r="CA6" t="inlineStr"/>
+      <c r="CB6" t="inlineStr"/>
+      <c r="CC6" t="inlineStr"/>
+      <c r="CD6" t="inlineStr"/>
+      <c r="CE6" t="inlineStr"/>
+      <c r="CF6" t="inlineStr"/>
+      <c r="CG6" t="inlineStr"/>
+      <c r="CH6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2016,6 +2086,13 @@
       <c r="BY7" t="inlineStr"/>
       <c r="BZ7" t="inlineStr"/>
       <c r="CA7" t="inlineStr"/>
+      <c r="CB7" t="inlineStr"/>
+      <c r="CC7" t="inlineStr"/>
+      <c r="CD7" t="inlineStr"/>
+      <c r="CE7" t="inlineStr"/>
+      <c r="CF7" t="inlineStr"/>
+      <c r="CG7" t="inlineStr"/>
+      <c r="CH7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2219,6 +2296,13 @@
       <c r="BY8" t="inlineStr"/>
       <c r="BZ8" t="inlineStr"/>
       <c r="CA8" t="inlineStr"/>
+      <c r="CB8" t="inlineStr"/>
+      <c r="CC8" t="inlineStr"/>
+      <c r="CD8" t="inlineStr"/>
+      <c r="CE8" t="inlineStr"/>
+      <c r="CF8" t="inlineStr"/>
+      <c r="CG8" t="inlineStr"/>
+      <c r="CH8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2424,6 +2508,13 @@
       <c r="BY9" t="inlineStr"/>
       <c r="BZ9" t="inlineStr"/>
       <c r="CA9" t="inlineStr"/>
+      <c r="CB9" t="inlineStr"/>
+      <c r="CC9" t="inlineStr"/>
+      <c r="CD9" t="inlineStr"/>
+      <c r="CE9" t="inlineStr"/>
+      <c r="CF9" t="inlineStr"/>
+      <c r="CG9" t="inlineStr"/>
+      <c r="CH9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2629,6 +2720,13 @@
       <c r="BY10" t="inlineStr"/>
       <c r="BZ10" t="inlineStr"/>
       <c r="CA10" t="inlineStr"/>
+      <c r="CB10" t="inlineStr"/>
+      <c r="CC10" t="inlineStr"/>
+      <c r="CD10" t="inlineStr"/>
+      <c r="CE10" t="inlineStr"/>
+      <c r="CF10" t="inlineStr"/>
+      <c r="CG10" t="inlineStr"/>
+      <c r="CH10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2833,6 +2931,13 @@
       <c r="BY11" t="inlineStr"/>
       <c r="BZ11" t="inlineStr"/>
       <c r="CA11" t="inlineStr"/>
+      <c r="CB11" t="inlineStr"/>
+      <c r="CC11" t="inlineStr"/>
+      <c r="CD11" t="inlineStr"/>
+      <c r="CE11" t="inlineStr"/>
+      <c r="CF11" t="inlineStr"/>
+      <c r="CG11" t="inlineStr"/>
+      <c r="CH11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3041,6 +3146,13 @@
       <c r="BY12" t="inlineStr"/>
       <c r="BZ12" t="inlineStr"/>
       <c r="CA12" t="inlineStr"/>
+      <c r="CB12" t="inlineStr"/>
+      <c r="CC12" t="inlineStr"/>
+      <c r="CD12" t="inlineStr"/>
+      <c r="CE12" t="inlineStr"/>
+      <c r="CF12" t="inlineStr"/>
+      <c r="CG12" t="inlineStr"/>
+      <c r="CH12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3245,6 +3357,13 @@
       <c r="BY13" t="inlineStr"/>
       <c r="BZ13" t="inlineStr"/>
       <c r="CA13" t="inlineStr"/>
+      <c r="CB13" t="inlineStr"/>
+      <c r="CC13" t="inlineStr"/>
+      <c r="CD13" t="inlineStr"/>
+      <c r="CE13" t="inlineStr"/>
+      <c r="CF13" t="inlineStr"/>
+      <c r="CG13" t="inlineStr"/>
+      <c r="CH13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3438,6 +3557,13 @@
       <c r="BY14" t="inlineStr"/>
       <c r="BZ14" t="inlineStr"/>
       <c r="CA14" t="inlineStr"/>
+      <c r="CB14" t="inlineStr"/>
+      <c r="CC14" t="inlineStr"/>
+      <c r="CD14" t="inlineStr"/>
+      <c r="CE14" t="inlineStr"/>
+      <c r="CF14" t="inlineStr"/>
+      <c r="CG14" t="inlineStr"/>
+      <c r="CH14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3640,6 +3766,13 @@
       <c r="BY15" t="inlineStr"/>
       <c r="BZ15" t="inlineStr"/>
       <c r="CA15" t="inlineStr"/>
+      <c r="CB15" t="inlineStr"/>
+      <c r="CC15" t="inlineStr"/>
+      <c r="CD15" t="inlineStr"/>
+      <c r="CE15" t="inlineStr"/>
+      <c r="CF15" t="inlineStr"/>
+      <c r="CG15" t="inlineStr"/>
+      <c r="CH15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3838,6 +3971,13 @@
       <c r="BY16" t="inlineStr"/>
       <c r="BZ16" t="inlineStr"/>
       <c r="CA16" t="inlineStr"/>
+      <c r="CB16" t="inlineStr"/>
+      <c r="CC16" t="inlineStr"/>
+      <c r="CD16" t="inlineStr"/>
+      <c r="CE16" t="inlineStr"/>
+      <c r="CF16" t="inlineStr"/>
+      <c r="CG16" t="inlineStr"/>
+      <c r="CH16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
@@ -3959,6 +4099,13 @@
       <c r="BY17" t="inlineStr"/>
       <c r="BZ17" t="inlineStr"/>
       <c r="CA17" t="inlineStr"/>
+      <c r="CB17" t="inlineStr"/>
+      <c r="CC17" t="inlineStr"/>
+      <c r="CD17" t="inlineStr"/>
+      <c r="CE17" t="inlineStr"/>
+      <c r="CF17" t="inlineStr"/>
+      <c r="CG17" t="inlineStr"/>
+      <c r="CH17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4130,6 +4277,13 @@
       <c r="BY18" t="inlineStr"/>
       <c r="BZ18" t="inlineStr"/>
       <c r="CA18" t="inlineStr"/>
+      <c r="CB18" t="inlineStr"/>
+      <c r="CC18" t="inlineStr"/>
+      <c r="CD18" t="inlineStr"/>
+      <c r="CE18" t="inlineStr"/>
+      <c r="CF18" t="inlineStr"/>
+      <c r="CG18" t="inlineStr"/>
+      <c r="CH18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4307,6 +4461,13 @@
       <c r="BY19" t="inlineStr"/>
       <c r="BZ19" t="inlineStr"/>
       <c r="CA19" t="inlineStr"/>
+      <c r="CB19" t="inlineStr"/>
+      <c r="CC19" t="inlineStr"/>
+      <c r="CD19" t="inlineStr"/>
+      <c r="CE19" t="inlineStr"/>
+      <c r="CF19" t="inlineStr"/>
+      <c r="CG19" t="inlineStr"/>
+      <c r="CH19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4340,35 +4501,23 @@
           <t>07:00</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>4009</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>848</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>3161</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>199</t>
-        </is>
+      <c r="H20" t="n">
+        <v>7</v>
+      </c>
+      <c r="I20" t="n">
+        <v>4009</v>
+      </c>
+      <c r="J20" t="n">
+        <v>848</v>
+      </c>
+      <c r="K20" t="n">
+        <v>30</v>
+      </c>
+      <c r="L20" t="n">
+        <v>3161</v>
+      </c>
+      <c r="M20" t="n">
+        <v>199</v>
       </c>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
@@ -4382,95 +4531,59 @@
           <t>0,90x4mm</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
-      </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>550</t>
-        </is>
-      </c>
-      <c r="W20" t="inlineStr">
-        <is>
-          <t>387</t>
-        </is>
-      </c>
-      <c r="X20" t="inlineStr">
-        <is>
-          <t>52</t>
-        </is>
-      </c>
-      <c r="Y20" t="inlineStr">
-        <is>
-          <t>725</t>
-        </is>
-      </c>
-      <c r="Z20" t="inlineStr">
-        <is>
-          <t>554</t>
-        </is>
-      </c>
-      <c r="AA20" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="AB20" t="inlineStr">
-        <is>
-          <t>840</t>
-        </is>
-      </c>
-      <c r="AC20" t="inlineStr">
-        <is>
-          <t>695</t>
-        </is>
-      </c>
-      <c r="AD20" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="AE20" t="inlineStr">
-        <is>
-          <t>530</t>
-        </is>
-      </c>
-      <c r="AF20" t="inlineStr">
-        <is>
-          <t>372</t>
-        </is>
-      </c>
-      <c r="AG20" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AH20" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AI20" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="R20" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" t="n">
+        <v>8</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" t="n">
+        <v>48</v>
+      </c>
+      <c r="V20" t="n">
+        <v>550</v>
+      </c>
+      <c r="W20" t="n">
+        <v>387</v>
+      </c>
+      <c r="X20" t="n">
+        <v>52</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>725</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>554</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>45</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>840</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>695</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>42</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>530</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>372</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>2</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
@@ -4512,48 +4625,32 @@
       </c>
       <c r="AT20" t="inlineStr"/>
       <c r="AU20" t="inlineStr"/>
-      <c r="AV20" t="inlineStr">
-        <is>
-          <t>800</t>
-        </is>
-      </c>
-      <c r="AW20" t="inlineStr">
-        <is>
-          <t>600</t>
-        </is>
+      <c r="AV20" t="n">
+        <v>800</v>
+      </c>
+      <c r="AW20" t="n">
+        <v>600</v>
       </c>
       <c r="AX20" t="inlineStr"/>
-      <c r="AY20" t="inlineStr">
-        <is>
-          <t>1400</t>
-        </is>
-      </c>
-      <c r="AZ20" t="inlineStr">
-        <is>
-          <t>744</t>
-        </is>
+      <c r="AY20" t="n">
+        <v>1400</v>
+      </c>
+      <c r="AZ20" t="n">
+        <v>744</v>
       </c>
       <c r="BA20" t="inlineStr"/>
-      <c r="BB20" t="inlineStr">
-        <is>
-          <t>1100</t>
-        </is>
-      </c>
-      <c r="BC20" t="inlineStr">
-        <is>
-          <t>657</t>
-        </is>
+      <c r="BB20" t="n">
+        <v>1100</v>
+      </c>
+      <c r="BC20" t="n">
+        <v>657</v>
       </c>
       <c r="BD20" t="inlineStr"/>
-      <c r="BE20" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BF20" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="BE20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF20" t="n">
+        <v>0</v>
       </c>
       <c r="BG20" t="inlineStr"/>
       <c r="BH20" t="inlineStr"/>
@@ -4596,6 +4693,177 @@
           <t>on</t>
         </is>
       </c>
+      <c r="CB20" t="inlineStr"/>
+      <c r="CC20" t="inlineStr"/>
+      <c r="CD20" t="inlineStr"/>
+      <c r="CE20" t="inlineStr"/>
+      <c r="CF20" t="inlineStr"/>
+      <c r="CG20" t="inlineStr"/>
+      <c r="CH20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="inlineStr"/>
+      <c r="AG21" t="inlineStr"/>
+      <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr"/>
+      <c r="AJ21" t="inlineStr"/>
+      <c r="AK21" t="inlineStr"/>
+      <c r="AL21" t="inlineStr"/>
+      <c r="AM21" t="inlineStr"/>
+      <c r="AN21" t="inlineStr"/>
+      <c r="AO21" t="inlineStr"/>
+      <c r="AP21" t="inlineStr"/>
+      <c r="AQ21" t="inlineStr"/>
+      <c r="AR21" t="inlineStr"/>
+      <c r="AS21" t="inlineStr"/>
+      <c r="AT21" t="inlineStr"/>
+      <c r="AU21" t="inlineStr"/>
+      <c r="AV21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX21" t="inlineStr"/>
+      <c r="AY21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA21" t="inlineStr"/>
+      <c r="BB21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD21" t="inlineStr"/>
+      <c r="BE21" t="inlineStr"/>
+      <c r="BF21" t="inlineStr"/>
+      <c r="BG21" t="inlineStr"/>
+      <c r="BH21" t="inlineStr"/>
+      <c r="BI21" t="inlineStr">
+        <is>
+          <t>11/06/2025</t>
+        </is>
+      </c>
+      <c r="BJ21" t="inlineStr">
+        <is>
+          <t>Teste Backup Automatico</t>
+        </is>
+      </c>
+      <c r="BK21" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="BL21" t="inlineStr">
+        <is>
+          <t>Dr. Teste</t>
+        </is>
+      </c>
+      <c r="BM21" t="inlineStr">
+        <is>
+          <t>Equipe Teste</t>
+        </is>
+      </c>
+      <c r="BN21" t="inlineStr"/>
+      <c r="BO21" t="inlineStr"/>
+      <c r="BP21" t="inlineStr">
+        <is>
+          <t>2500</t>
+        </is>
+      </c>
+      <c r="BQ21" t="inlineStr">
+        <is>
+          <t>800</t>
+        </is>
+      </c>
+      <c r="BR21" t="inlineStr"/>
+      <c r="BS21" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="BT21" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="BU21" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="BV21" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="BW21" t="inlineStr"/>
+      <c r="BX21" t="inlineStr"/>
+      <c r="BY21" t="inlineStr"/>
+      <c r="BZ21" t="inlineStr"/>
+      <c r="CA21" t="inlineStr"/>
+      <c r="CB21" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="CC21" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="CD21" t="inlineStr">
+        <is>
+          <t>85.5</t>
+        </is>
+      </c>
+      <c r="CE21" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="CF21" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG21" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update surgical summary to include all registered data
Attach a comprehensive surgical summary report to the system, incorporating all collected patient and procedural details.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 7910296b-13ef-440a-bc5d-2363bc1496e5
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/8c7417ff-25e3-4894-9a88-ca4d88413804/7910296b-13ef-440a-bc5d-2363bc1496e5/FeXtGVh
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CH21"/>
+  <dimension ref="A1:CP22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -857,6 +857,46 @@
       <c r="CH1" s="1" t="inlineStr">
         <is>
           <t>pernas_comentarios</t>
+        </is>
+      </c>
+      <c r="CI1" s="1" t="inlineStr">
+        <is>
+          <t>q1_densidade</t>
+        </is>
+      </c>
+      <c r="CJ1" s="1" t="inlineStr">
+        <is>
+          <t>q1_taxa_quebra</t>
+        </is>
+      </c>
+      <c r="CK1" s="1" t="inlineStr">
+        <is>
+          <t>q2_densidade</t>
+        </is>
+      </c>
+      <c r="CL1" s="1" t="inlineStr">
+        <is>
+          <t>q2_taxa_quebra</t>
+        </is>
+      </c>
+      <c r="CM1" s="1" t="inlineStr">
+        <is>
+          <t>q3_densidade</t>
+        </is>
+      </c>
+      <c r="CN1" s="1" t="inlineStr">
+        <is>
+          <t>q3_taxa_quebra</t>
+        </is>
+      </c>
+      <c r="CO1" s="1" t="inlineStr">
+        <is>
+          <t>q4_densidade</t>
+        </is>
+      </c>
+      <c r="CP1" s="1" t="inlineStr">
+        <is>
+          <t>q4_taxa_quebra</t>
         </is>
       </c>
     </row>
@@ -1053,6 +1093,14 @@
       <c r="CF2" t="inlineStr"/>
       <c r="CG2" t="inlineStr"/>
       <c r="CH2" t="inlineStr"/>
+      <c r="CI2" t="inlineStr"/>
+      <c r="CJ2" t="inlineStr"/>
+      <c r="CK2" t="inlineStr"/>
+      <c r="CL2" t="inlineStr"/>
+      <c r="CM2" t="inlineStr"/>
+      <c r="CN2" t="inlineStr"/>
+      <c r="CO2" t="inlineStr"/>
+      <c r="CP2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1257,6 +1305,14 @@
       <c r="CF3" t="inlineStr"/>
       <c r="CG3" t="inlineStr"/>
       <c r="CH3" t="inlineStr"/>
+      <c r="CI3" t="inlineStr"/>
+      <c r="CJ3" t="inlineStr"/>
+      <c r="CK3" t="inlineStr"/>
+      <c r="CL3" t="inlineStr"/>
+      <c r="CM3" t="inlineStr"/>
+      <c r="CN3" t="inlineStr"/>
+      <c r="CO3" t="inlineStr"/>
+      <c r="CP3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1466,6 +1522,14 @@
       <c r="CF4" t="inlineStr"/>
       <c r="CG4" t="inlineStr"/>
       <c r="CH4" t="inlineStr"/>
+      <c r="CI4" t="inlineStr"/>
+      <c r="CJ4" t="inlineStr"/>
+      <c r="CK4" t="inlineStr"/>
+      <c r="CL4" t="inlineStr"/>
+      <c r="CM4" t="inlineStr"/>
+      <c r="CN4" t="inlineStr"/>
+      <c r="CO4" t="inlineStr"/>
+      <c r="CP4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1670,6 +1734,14 @@
       <c r="CF5" t="inlineStr"/>
       <c r="CG5" t="inlineStr"/>
       <c r="CH5" t="inlineStr"/>
+      <c r="CI5" t="inlineStr"/>
+      <c r="CJ5" t="inlineStr"/>
+      <c r="CK5" t="inlineStr"/>
+      <c r="CL5" t="inlineStr"/>
+      <c r="CM5" t="inlineStr"/>
+      <c r="CN5" t="inlineStr"/>
+      <c r="CO5" t="inlineStr"/>
+      <c r="CP5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1878,6 +1950,14 @@
       <c r="CF6" t="inlineStr"/>
       <c r="CG6" t="inlineStr"/>
       <c r="CH6" t="inlineStr"/>
+      <c r="CI6" t="inlineStr"/>
+      <c r="CJ6" t="inlineStr"/>
+      <c r="CK6" t="inlineStr"/>
+      <c r="CL6" t="inlineStr"/>
+      <c r="CM6" t="inlineStr"/>
+      <c r="CN6" t="inlineStr"/>
+      <c r="CO6" t="inlineStr"/>
+      <c r="CP6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2093,6 +2173,14 @@
       <c r="CF7" t="inlineStr"/>
       <c r="CG7" t="inlineStr"/>
       <c r="CH7" t="inlineStr"/>
+      <c r="CI7" t="inlineStr"/>
+      <c r="CJ7" t="inlineStr"/>
+      <c r="CK7" t="inlineStr"/>
+      <c r="CL7" t="inlineStr"/>
+      <c r="CM7" t="inlineStr"/>
+      <c r="CN7" t="inlineStr"/>
+      <c r="CO7" t="inlineStr"/>
+      <c r="CP7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2303,6 +2391,14 @@
       <c r="CF8" t="inlineStr"/>
       <c r="CG8" t="inlineStr"/>
       <c r="CH8" t="inlineStr"/>
+      <c r="CI8" t="inlineStr"/>
+      <c r="CJ8" t="inlineStr"/>
+      <c r="CK8" t="inlineStr"/>
+      <c r="CL8" t="inlineStr"/>
+      <c r="CM8" t="inlineStr"/>
+      <c r="CN8" t="inlineStr"/>
+      <c r="CO8" t="inlineStr"/>
+      <c r="CP8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2515,6 +2611,14 @@
       <c r="CF9" t="inlineStr"/>
       <c r="CG9" t="inlineStr"/>
       <c r="CH9" t="inlineStr"/>
+      <c r="CI9" t="inlineStr"/>
+      <c r="CJ9" t="inlineStr"/>
+      <c r="CK9" t="inlineStr"/>
+      <c r="CL9" t="inlineStr"/>
+      <c r="CM9" t="inlineStr"/>
+      <c r="CN9" t="inlineStr"/>
+      <c r="CO9" t="inlineStr"/>
+      <c r="CP9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2727,6 +2831,14 @@
       <c r="CF10" t="inlineStr"/>
       <c r="CG10" t="inlineStr"/>
       <c r="CH10" t="inlineStr"/>
+      <c r="CI10" t="inlineStr"/>
+      <c r="CJ10" t="inlineStr"/>
+      <c r="CK10" t="inlineStr"/>
+      <c r="CL10" t="inlineStr"/>
+      <c r="CM10" t="inlineStr"/>
+      <c r="CN10" t="inlineStr"/>
+      <c r="CO10" t="inlineStr"/>
+      <c r="CP10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2938,6 +3050,14 @@
       <c r="CF11" t="inlineStr"/>
       <c r="CG11" t="inlineStr"/>
       <c r="CH11" t="inlineStr"/>
+      <c r="CI11" t="inlineStr"/>
+      <c r="CJ11" t="inlineStr"/>
+      <c r="CK11" t="inlineStr"/>
+      <c r="CL11" t="inlineStr"/>
+      <c r="CM11" t="inlineStr"/>
+      <c r="CN11" t="inlineStr"/>
+      <c r="CO11" t="inlineStr"/>
+      <c r="CP11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3153,6 +3273,14 @@
       <c r="CF12" t="inlineStr"/>
       <c r="CG12" t="inlineStr"/>
       <c r="CH12" t="inlineStr"/>
+      <c r="CI12" t="inlineStr"/>
+      <c r="CJ12" t="inlineStr"/>
+      <c r="CK12" t="inlineStr"/>
+      <c r="CL12" t="inlineStr"/>
+      <c r="CM12" t="inlineStr"/>
+      <c r="CN12" t="inlineStr"/>
+      <c r="CO12" t="inlineStr"/>
+      <c r="CP12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3364,6 +3492,14 @@
       <c r="CF13" t="inlineStr"/>
       <c r="CG13" t="inlineStr"/>
       <c r="CH13" t="inlineStr"/>
+      <c r="CI13" t="inlineStr"/>
+      <c r="CJ13" t="inlineStr"/>
+      <c r="CK13" t="inlineStr"/>
+      <c r="CL13" t="inlineStr"/>
+      <c r="CM13" t="inlineStr"/>
+      <c r="CN13" t="inlineStr"/>
+      <c r="CO13" t="inlineStr"/>
+      <c r="CP13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3564,6 +3700,14 @@
       <c r="CF14" t="inlineStr"/>
       <c r="CG14" t="inlineStr"/>
       <c r="CH14" t="inlineStr"/>
+      <c r="CI14" t="inlineStr"/>
+      <c r="CJ14" t="inlineStr"/>
+      <c r="CK14" t="inlineStr"/>
+      <c r="CL14" t="inlineStr"/>
+      <c r="CM14" t="inlineStr"/>
+      <c r="CN14" t="inlineStr"/>
+      <c r="CO14" t="inlineStr"/>
+      <c r="CP14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3773,6 +3917,14 @@
       <c r="CF15" t="inlineStr"/>
       <c r="CG15" t="inlineStr"/>
       <c r="CH15" t="inlineStr"/>
+      <c r="CI15" t="inlineStr"/>
+      <c r="CJ15" t="inlineStr"/>
+      <c r="CK15" t="inlineStr"/>
+      <c r="CL15" t="inlineStr"/>
+      <c r="CM15" t="inlineStr"/>
+      <c r="CN15" t="inlineStr"/>
+      <c r="CO15" t="inlineStr"/>
+      <c r="CP15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3978,6 +4130,14 @@
       <c r="CF16" t="inlineStr"/>
       <c r="CG16" t="inlineStr"/>
       <c r="CH16" t="inlineStr"/>
+      <c r="CI16" t="inlineStr"/>
+      <c r="CJ16" t="inlineStr"/>
+      <c r="CK16" t="inlineStr"/>
+      <c r="CL16" t="inlineStr"/>
+      <c r="CM16" t="inlineStr"/>
+      <c r="CN16" t="inlineStr"/>
+      <c r="CO16" t="inlineStr"/>
+      <c r="CP16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
@@ -4106,6 +4266,14 @@
       <c r="CF17" t="inlineStr"/>
       <c r="CG17" t="inlineStr"/>
       <c r="CH17" t="inlineStr"/>
+      <c r="CI17" t="inlineStr"/>
+      <c r="CJ17" t="inlineStr"/>
+      <c r="CK17" t="inlineStr"/>
+      <c r="CL17" t="inlineStr"/>
+      <c r="CM17" t="inlineStr"/>
+      <c r="CN17" t="inlineStr"/>
+      <c r="CO17" t="inlineStr"/>
+      <c r="CP17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4284,6 +4452,14 @@
       <c r="CF18" t="inlineStr"/>
       <c r="CG18" t="inlineStr"/>
       <c r="CH18" t="inlineStr"/>
+      <c r="CI18" t="inlineStr"/>
+      <c r="CJ18" t="inlineStr"/>
+      <c r="CK18" t="inlineStr"/>
+      <c r="CL18" t="inlineStr"/>
+      <c r="CM18" t="inlineStr"/>
+      <c r="CN18" t="inlineStr"/>
+      <c r="CO18" t="inlineStr"/>
+      <c r="CP18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4468,6 +4644,14 @@
       <c r="CF19" t="inlineStr"/>
       <c r="CG19" t="inlineStr"/>
       <c r="CH19" t="inlineStr"/>
+      <c r="CI19" t="inlineStr"/>
+      <c r="CJ19" t="inlineStr"/>
+      <c r="CK19" t="inlineStr"/>
+      <c r="CL19" t="inlineStr"/>
+      <c r="CM19" t="inlineStr"/>
+      <c r="CN19" t="inlineStr"/>
+      <c r="CO19" t="inlineStr"/>
+      <c r="CP19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4700,6 +4884,14 @@
       <c r="CF20" t="inlineStr"/>
       <c r="CG20" t="inlineStr"/>
       <c r="CH20" t="inlineStr"/>
+      <c r="CI20" t="inlineStr"/>
+      <c r="CJ20" t="inlineStr"/>
+      <c r="CK20" t="inlineStr"/>
+      <c r="CL20" t="inlineStr"/>
+      <c r="CM20" t="inlineStr"/>
+      <c r="CN20" t="inlineStr"/>
+      <c r="CO20" t="inlineStr"/>
+      <c r="CP20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
@@ -4801,36 +4993,24 @@
       </c>
       <c r="BN21" t="inlineStr"/>
       <c r="BO21" t="inlineStr"/>
-      <c r="BP21" t="inlineStr">
-        <is>
-          <t>2500</t>
-        </is>
-      </c>
-      <c r="BQ21" t="inlineStr">
-        <is>
-          <t>800</t>
-        </is>
+      <c r="BP21" t="n">
+        <v>2500</v>
+      </c>
+      <c r="BQ21" t="n">
+        <v>800</v>
       </c>
       <c r="BR21" t="inlineStr"/>
-      <c r="BS21" t="inlineStr">
-        <is>
-          <t>600</t>
-        </is>
-      </c>
-      <c r="BT21" t="inlineStr">
-        <is>
-          <t>400</t>
-        </is>
-      </c>
-      <c r="BU21" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-      <c r="BV21" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
+      <c r="BS21" t="n">
+        <v>600</v>
+      </c>
+      <c r="BT21" t="n">
+        <v>400</v>
+      </c>
+      <c r="BU21" t="n">
+        <v>350</v>
+      </c>
+      <c r="BV21" t="n">
+        <v>350</v>
       </c>
       <c r="BW21" t="inlineStr"/>
       <c r="BX21" t="inlineStr"/>
@@ -4842,15 +5022,11 @@
           <t>10:30</t>
         </is>
       </c>
-      <c r="CC21" t="inlineStr">
-        <is>
-          <t>3.5</t>
-        </is>
-      </c>
-      <c r="CD21" t="inlineStr">
-        <is>
-          <t>85.5</t>
-        </is>
+      <c r="CC21" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="CD21" t="n">
+        <v>85.5</v>
       </c>
       <c r="CE21" t="inlineStr">
         <is>
@@ -4864,6 +5040,330 @@
         <v>0</v>
       </c>
       <c r="CH21" t="inlineStr"/>
+      <c r="CI21" t="inlineStr"/>
+      <c r="CJ21" t="inlineStr"/>
+      <c r="CK21" t="inlineStr"/>
+      <c r="CL21" t="inlineStr"/>
+      <c r="CM21" t="inlineStr"/>
+      <c r="CN21" t="inlineStr"/>
+      <c r="CO21" t="inlineStr"/>
+      <c r="CP21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025-08-20</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>teste1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Dr. Arthur</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Aline, Ana, Lavinia, Natália, Aline, Ana, Lavinia, Natália</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>0,85x3,5mm</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AI22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AK22" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL22" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AM22" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN22" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>ndn</t>
+        </is>
+      </c>
+      <c r="AP22" t="inlineStr">
+        <is>
+          <t>fios finos</t>
+        </is>
+      </c>
+      <c r="AQ22" t="inlineStr"/>
+      <c r="AR22" t="inlineStr"/>
+      <c r="AS22" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT22" t="inlineStr"/>
+      <c r="AU22" t="inlineStr"/>
+      <c r="AV22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX22" t="inlineStr"/>
+      <c r="AY22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA22" t="inlineStr"/>
+      <c r="BB22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD22" t="inlineStr"/>
+      <c r="BE22" t="inlineStr"/>
+      <c r="BF22" t="inlineStr"/>
+      <c r="BG22" t="inlineStr"/>
+      <c r="BH22" t="inlineStr"/>
+      <c r="BI22" t="inlineStr"/>
+      <c r="BJ22" t="inlineStr"/>
+      <c r="BK22" t="inlineStr"/>
+      <c r="BL22" t="inlineStr"/>
+      <c r="BM22" t="inlineStr"/>
+      <c r="BN22" t="inlineStr"/>
+      <c r="BO22" t="inlineStr"/>
+      <c r="BP22" t="inlineStr"/>
+      <c r="BQ22" t="inlineStr"/>
+      <c r="BR22" t="inlineStr"/>
+      <c r="BS22" t="inlineStr"/>
+      <c r="BT22" t="inlineStr"/>
+      <c r="BU22" t="inlineStr"/>
+      <c r="BV22" t="inlineStr"/>
+      <c r="BW22" t="inlineStr"/>
+      <c r="BX22" t="inlineStr"/>
+      <c r="BY22" t="inlineStr"/>
+      <c r="BZ22" t="inlineStr"/>
+      <c r="CA22" t="inlineStr"/>
+      <c r="CB22" t="inlineStr"/>
+      <c r="CC22" t="inlineStr"/>
+      <c r="CD22" t="inlineStr"/>
+      <c r="CE22" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="CF22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH22" t="inlineStr"/>
+      <c r="CI22" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="CJ22" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="CK22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="CL22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="CM22" t="inlineStr">
+        <is>
+          <t>0.40816326530612246</t>
+        </is>
+      </c>
+      <c r="CN22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="CO22" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="CP22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Remove unused patient data fields from success page display
Remove 'Idade', 'Sexo', and 'Técnica' fields from the success.html template and correct date formatting logic.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 7910296b-13ef-440a-bc5d-2363bc1496e5
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/8c7417ff-25e3-4894-9a88-ca4d88413804/7910296b-13ef-440a-bc5d-2363bc1496e5/6Ca0D35
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CP22"/>
+  <dimension ref="A1:CP23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5081,45 +5081,29 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
+      <c r="H22" t="n">
+        <v>5</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" t="n">
+        <v>20</v>
+      </c>
+      <c r="K22" t="n">
+        <v>20</v>
+      </c>
+      <c r="L22" t="n">
+        <v>20</v>
+      </c>
+      <c r="M22" t="n">
+        <v>20</v>
+      </c>
+      <c r="N22" t="n">
+        <v>24</v>
+      </c>
+      <c r="O22" t="n">
+        <v>23</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
@@ -5131,95 +5115,59 @@
           <t>0,85x3,5mm</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>54</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="X22" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="Y22" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="Z22" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="AA22" t="inlineStr">
-        <is>
-          <t>49</t>
-        </is>
-      </c>
-      <c r="AB22" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="AC22" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="AD22" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="AE22" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="AF22" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="AG22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AH22" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AI22" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="R22" t="n">
+        <v>23</v>
+      </c>
+      <c r="S22" t="n">
+        <v>23</v>
+      </c>
+      <c r="T22" t="n">
+        <v>54</v>
+      </c>
+      <c r="U22" t="n">
+        <v>50</v>
+      </c>
+      <c r="V22" t="n">
+        <v>10</v>
+      </c>
+      <c r="W22" t="n">
+        <v>8</v>
+      </c>
+      <c r="X22" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>19</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>19</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>49</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>20</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>20</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>50</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>40</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>40</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH22" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>2</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
@@ -5324,44 +5272,344 @@
         <v>0</v>
       </c>
       <c r="CH22" t="inlineStr"/>
-      <c r="CI22" t="inlineStr">
-        <is>
-          <t>0.2</t>
-        </is>
-      </c>
-      <c r="CJ22" t="inlineStr">
-        <is>
-          <t>0.2</t>
-        </is>
-      </c>
-      <c r="CK22" t="inlineStr">
+      <c r="CI22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="CJ22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="CK22" t="n">
+        <v>1</v>
+      </c>
+      <c r="CL22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM22" t="n">
+        <v>0.4081632653061224</v>
+      </c>
+      <c r="CN22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO22" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="CP22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2025-08-06</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>teste1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Dr. Daniel</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Ana, Ana</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>0,85x4mm</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="CL22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="CM22" t="inlineStr">
-        <is>
-          <t>0.40816326530612246</t>
-        </is>
-      </c>
-      <c r="CN22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="CO22" t="inlineStr">
-        <is>
-          <t>0.8</t>
-        </is>
-      </c>
-      <c r="CP22" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AI23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AL23" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM23" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>ndn</t>
+        </is>
+      </c>
+      <c r="AP23" t="inlineStr">
+        <is>
+          <t>fios finos</t>
+        </is>
+      </c>
+      <c r="AQ23" t="inlineStr"/>
+      <c r="AR23" t="inlineStr"/>
+      <c r="AS23" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT23" t="inlineStr"/>
+      <c r="AU23" t="inlineStr"/>
+      <c r="AV23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX23" t="inlineStr"/>
+      <c r="AY23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA23" t="inlineStr"/>
+      <c r="BB23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD23" t="inlineStr"/>
+      <c r="BE23" t="inlineStr"/>
+      <c r="BF23" t="inlineStr"/>
+      <c r="BG23" t="inlineStr"/>
+      <c r="BH23" t="inlineStr"/>
+      <c r="BI23" t="inlineStr"/>
+      <c r="BJ23" t="inlineStr"/>
+      <c r="BK23" t="inlineStr"/>
+      <c r="BL23" t="inlineStr"/>
+      <c r="BM23" t="inlineStr"/>
+      <c r="BN23" t="inlineStr"/>
+      <c r="BO23" t="inlineStr"/>
+      <c r="BP23" t="inlineStr"/>
+      <c r="BQ23" t="inlineStr"/>
+      <c r="BR23" t="inlineStr"/>
+      <c r="BS23" t="inlineStr"/>
+      <c r="BT23" t="inlineStr"/>
+      <c r="BU23" t="inlineStr"/>
+      <c r="BV23" t="inlineStr"/>
+      <c r="BW23" t="inlineStr"/>
+      <c r="BX23" t="inlineStr"/>
+      <c r="BY23" t="inlineStr"/>
+      <c r="BZ23" t="inlineStr"/>
+      <c r="CA23" t="inlineStr"/>
+      <c r="CB23" t="inlineStr"/>
+      <c r="CC23" t="inlineStr"/>
+      <c r="CD23" t="inlineStr"/>
+      <c r="CE23" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="CF23" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG23" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH23" t="inlineStr"/>
+      <c r="CI23" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="CJ23" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="CK23" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="CL23" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="CM23" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="CN23" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="CO23" t="inlineStr">
+        <is>
+          <t>11.666666666666666</t>
+        </is>
+      </c>
+      <c r="CP23" t="inlineStr">
+        <is>
+          <t>0.9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update success page to display detailed body hair transplant information
Update the success template to conditionally display body hair data, including furos, fios, and comments for various body parts, alongside unique team member display.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 7910296b-13ef-440a-bc5d-2363bc1496e5
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/8c7417ff-25e3-4894-9a88-ca4d88413804/7910296b-13ef-440a-bc5d-2363bc1496e5/JP193ci
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CP23"/>
+  <dimension ref="A1:CP24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5329,45 +5329,29 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
+      <c r="H23" t="n">
+        <v>5</v>
+      </c>
+      <c r="I23" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J23" t="n">
+        <v>200</v>
+      </c>
+      <c r="K23" t="n">
+        <v>70</v>
+      </c>
+      <c r="L23" t="n">
+        <v>500</v>
+      </c>
+      <c r="M23" t="n">
+        <v>300</v>
+      </c>
+      <c r="N23" t="n">
+        <v>20</v>
+      </c>
+      <c r="O23" t="n">
+        <v>20</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
@@ -5379,95 +5363,59 @@
           <t>0,85x4mm</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="W23" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="Y23" t="inlineStr">
-        <is>
-          <t>400</t>
-        </is>
-      </c>
-      <c r="Z23" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="AA23" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="AB23" t="inlineStr">
-        <is>
-          <t>600</t>
-        </is>
-      </c>
-      <c r="AC23" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="AD23" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="AE23" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
-      </c>
-      <c r="AF23" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
-      <c r="AG23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AH23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AI23" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="R23" t="n">
+        <v>5</v>
+      </c>
+      <c r="S23" t="n">
+        <v>10</v>
+      </c>
+      <c r="T23" t="n">
+        <v>10</v>
+      </c>
+      <c r="U23" t="n">
+        <v>10</v>
+      </c>
+      <c r="V23" t="n">
+        <v>300</v>
+      </c>
+      <c r="W23" t="n">
+        <v>30</v>
+      </c>
+      <c r="X23" t="n">
+        <v>10</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>400</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>40</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>50</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>600</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>60</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>700</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>70</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>2</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
@@ -5572,44 +5520,336 @@
         <v>0</v>
       </c>
       <c r="CH23" t="inlineStr"/>
-      <c r="CI23" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="CJ23" t="inlineStr">
+      <c r="CI23" t="n">
+        <v>30</v>
+      </c>
+      <c r="CJ23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="CK23" t="n">
+        <v>40</v>
+      </c>
+      <c r="CL23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="CM23" t="n">
+        <v>12</v>
+      </c>
+      <c r="CN23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="CO23" t="n">
+        <v>11.66666666666667</v>
+      </c>
+      <c r="CP23" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2025-08-12</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>teste1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Dr. Daniel</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Técnica Extra 1: thamara, Técnica Extra 2: larissa, Ana, Lavinia, Técnica Extra 1: thamara, Técnica Extra 2: larissa, Ana, Lavinia, Técnica Extra 1: thamara, Técnica Extra 2: larissa</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>0,90x5mm</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AI24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK24" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL24" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM24" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN24" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AO24" t="inlineStr">
+        <is>
+          <t>NDN</t>
+        </is>
+      </c>
+      <c r="AP24" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AQ24" t="inlineStr">
+        <is>
+          <t>thamara</t>
+        </is>
+      </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>larissa</t>
+        </is>
+      </c>
+      <c r="AS24" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT24" t="inlineStr"/>
+      <c r="AU24" t="inlineStr"/>
+      <c r="AV24" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AW24" t="n">
+        <v>210</v>
+      </c>
+      <c r="AX24" t="inlineStr"/>
+      <c r="AY24" t="n">
+        <v>100</v>
+      </c>
+      <c r="AZ24" t="n">
+        <v>50</v>
+      </c>
+      <c r="BA24" t="inlineStr"/>
+      <c r="BB24" t="n">
+        <v>1200</v>
+      </c>
+      <c r="BC24" t="n">
+        <v>1000</v>
+      </c>
+      <c r="BD24" t="inlineStr"/>
+      <c r="BE24" t="inlineStr"/>
+      <c r="BF24" t="inlineStr"/>
+      <c r="BG24" t="inlineStr"/>
+      <c r="BH24" t="inlineStr"/>
+      <c r="BI24" t="inlineStr"/>
+      <c r="BJ24" t="inlineStr"/>
+      <c r="BK24" t="inlineStr"/>
+      <c r="BL24" t="inlineStr"/>
+      <c r="BM24" t="inlineStr"/>
+      <c r="BN24" t="inlineStr"/>
+      <c r="BO24" t="inlineStr"/>
+      <c r="BP24" t="inlineStr"/>
+      <c r="BQ24" t="inlineStr"/>
+      <c r="BR24" t="inlineStr"/>
+      <c r="BS24" t="inlineStr"/>
+      <c r="BT24" t="inlineStr"/>
+      <c r="BU24" t="inlineStr"/>
+      <c r="BV24" t="inlineStr"/>
+      <c r="BW24" t="inlineStr"/>
+      <c r="BX24" t="inlineStr"/>
+      <c r="BY24" t="inlineStr"/>
+      <c r="BZ24" t="inlineStr"/>
+      <c r="CA24" t="inlineStr"/>
+      <c r="CB24" t="inlineStr"/>
+      <c r="CC24" t="inlineStr"/>
+      <c r="CD24" t="inlineStr"/>
+      <c r="CE24" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="CF24" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG24" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH24" t="inlineStr"/>
+      <c r="CI24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="CJ24" t="inlineStr">
         <is>
           <t>0.9</t>
         </is>
       </c>
-      <c r="CK23" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="CL23" t="inlineStr">
+      <c r="CK24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="CL24" t="inlineStr">
         <is>
           <t>0.9</t>
         </is>
       </c>
-      <c r="CM23" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="CN23" t="inlineStr">
-        <is>
-          <t>0.9</t>
-        </is>
-      </c>
-      <c r="CO23" t="inlineStr">
-        <is>
-          <t>11.666666666666666</t>
-        </is>
-      </c>
-      <c r="CP23" t="inlineStr">
-        <is>
-          <t>0.9</t>
+      <c r="CM24" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="CN24" t="inlineStr">
+        <is>
+          <t>0.900990099009901</t>
+        </is>
+      </c>
+      <c r="CO24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="CP24" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update date format to Brazilian standard
Modify the success template to display dates in DD/MM/YYYY format, and create a backup of the surgery data.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 7910296b-13ef-440a-bc5d-2363bc1496e5
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/8c7417ff-25e3-4894-9a88-ca4d88413804/7910296b-13ef-440a-bc5d-2363bc1496e5/gQp39Yw
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CP24"/>
+  <dimension ref="A1:CP25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5577,30 +5577,20 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
+      <c r="H24" t="n">
+        <v>5</v>
+      </c>
+      <c r="I24" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J24" t="n">
+        <v>20</v>
+      </c>
+      <c r="K24" t="n">
+        <v>20</v>
+      </c>
+      <c r="L24" t="n">
+        <v>20</v>
       </c>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
@@ -5615,91 +5605,57 @@
           <t>0,90x5mm</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="R24" t="n">
+        <v>10</v>
       </c>
       <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="W24" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="X24" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="Y24" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="Z24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AA24" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AB24" t="inlineStr">
-        <is>
-          <t>101</t>
-        </is>
-      </c>
-      <c r="AC24" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AD24" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AE24" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AF24" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AG24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AH24" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AI24" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="T24" t="n">
+        <v>4</v>
+      </c>
+      <c r="U24" t="n">
+        <v>100</v>
+      </c>
+      <c r="V24" t="n">
+        <v>100</v>
+      </c>
+      <c r="W24" t="n">
+        <v>10</v>
+      </c>
+      <c r="X24" t="n">
+        <v>10</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>101</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>10</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI24" t="n">
+        <v>2</v>
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
@@ -5812,42 +5768,318 @@
         <v>0</v>
       </c>
       <c r="CH24" t="inlineStr"/>
-      <c r="CI24" t="inlineStr">
+      <c r="CI24" t="n">
+        <v>1</v>
+      </c>
+      <c r="CJ24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="CK24" t="n">
+        <v>1</v>
+      </c>
+      <c r="CL24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="CM24" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="CN24" t="n">
+        <v>0.900990099009901</v>
+      </c>
+      <c r="CO24" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2025-08-12</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>teste1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Dr. Arthur</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Técnica Extra 1: thamara, Técnica Extra 2: larissa, Aline, Ana, Lavinia, Natália, Técnica Extra 1: thamara, Técnica Extra 2: larissa, Aline, Ana, Lavinia, Natália, Técnica Extra 1: thamara, Técnica Extra 2: larissa</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>0,85x3,5mm</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="CJ24" t="inlineStr">
-        <is>
-          <t>0.9</t>
-        </is>
-      </c>
-      <c r="CK24" t="inlineStr">
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AI25" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="CL24" t="inlineStr">
-        <is>
-          <t>0.9</t>
-        </is>
-      </c>
-      <c r="CM24" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="CN24" t="inlineStr">
-        <is>
-          <t>0.900990099009901</t>
-        </is>
-      </c>
-      <c r="CO24" t="inlineStr">
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK25" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AL25" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AN25" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AO25" t="inlineStr">
+        <is>
+          <t>ndn</t>
+        </is>
+      </c>
+      <c r="AP25" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AQ25" t="inlineStr">
+        <is>
+          <t>thamara</t>
+        </is>
+      </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>larissa</t>
+        </is>
+      </c>
+      <c r="AS25" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AT25" t="inlineStr"/>
+      <c r="AU25" t="inlineStr"/>
+      <c r="AV25" t="n">
+        <v>100</v>
+      </c>
+      <c r="AW25" t="n">
+        <v>100</v>
+      </c>
+      <c r="AX25" t="inlineStr"/>
+      <c r="AY25" t="n">
+        <v>10</v>
+      </c>
+      <c r="AZ25" t="n">
+        <v>20</v>
+      </c>
+      <c r="BA25" t="inlineStr"/>
+      <c r="BB25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD25" t="inlineStr"/>
+      <c r="BE25" t="inlineStr"/>
+      <c r="BF25" t="inlineStr"/>
+      <c r="BG25" t="inlineStr"/>
+      <c r="BH25" t="inlineStr"/>
+      <c r="BI25" t="inlineStr"/>
+      <c r="BJ25" t="inlineStr"/>
+      <c r="BK25" t="inlineStr"/>
+      <c r="BL25" t="inlineStr"/>
+      <c r="BM25" t="inlineStr"/>
+      <c r="BN25" t="inlineStr"/>
+      <c r="BO25" t="inlineStr"/>
+      <c r="BP25" t="inlineStr"/>
+      <c r="BQ25" t="inlineStr"/>
+      <c r="BR25" t="inlineStr"/>
+      <c r="BS25" t="inlineStr"/>
+      <c r="BT25" t="inlineStr"/>
+      <c r="BU25" t="inlineStr"/>
+      <c r="BV25" t="inlineStr"/>
+      <c r="BW25" t="inlineStr"/>
+      <c r="BX25" t="inlineStr"/>
+      <c r="BY25" t="inlineStr"/>
+      <c r="BZ25" t="inlineStr"/>
+      <c r="CA25" t="inlineStr"/>
+      <c r="CB25" t="inlineStr"/>
+      <c r="CC25" t="inlineStr"/>
+      <c r="CD25" t="inlineStr"/>
+      <c r="CE25" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="CF25" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG25" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH25" t="inlineStr"/>
+      <c r="CI25" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="CP24" t="inlineStr">
+      <c r="CJ25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="CK25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="CL25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="CM25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="CN25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="CO25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="CP25" t="inlineStr">
         <is>
           <t>0</t>
         </is>

</xml_diff>

<commit_message>
Improve accuracy of duplicate surgery checks by normalizing names
Refactor the `check_duplicate_surgery` function in `app.py` to normalize patient names using `.strip().upper()` before comparison, ensuring more reliable duplicate detection and preventing false positives.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 509a755b-bfe1-4381-9dd3-19cabc1fcee4
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Event-Id: 9225f357-6845-4dd1-89a4-fd13a2a4e426
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/8c7417ff-25e3-4894-9a88-ca4d88413804/509a755b-bfe1-4381-9dd3-19cabc1fcee4/UFPIanA
</commit_message>
<xml_diff>
--- a/cirurgias.xlsx
+++ b/cirurgias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ26"/>
+  <dimension ref="A1:CT29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -902,6 +902,21 @@
       <c r="CQ1" s="1" t="inlineStr">
         <is>
           <t>extra_person_3</t>
+        </is>
+      </c>
+      <c r="CR1" s="1" t="inlineStr">
+        <is>
+          <t>tecnica</t>
+        </is>
+      </c>
+      <c r="CS1" s="1" t="inlineStr">
+        <is>
+          <t>tipo_implante</t>
+        </is>
+      </c>
+      <c r="CT1" s="1" t="inlineStr">
+        <is>
+          <t>retoque</t>
         </is>
       </c>
     </row>
@@ -1107,6 +1122,9 @@
       <c r="CO2" t="inlineStr"/>
       <c r="CP2" t="inlineStr"/>
       <c r="CQ2" t="inlineStr"/>
+      <c r="CR2" t="inlineStr"/>
+      <c r="CS2" t="inlineStr"/>
+      <c r="CT2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1320,6 +1338,9 @@
       <c r="CO3" t="inlineStr"/>
       <c r="CP3" t="inlineStr"/>
       <c r="CQ3" t="inlineStr"/>
+      <c r="CR3" t="inlineStr"/>
+      <c r="CS3" t="inlineStr"/>
+      <c r="CT3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1538,6 +1559,9 @@
       <c r="CO4" t="inlineStr"/>
       <c r="CP4" t="inlineStr"/>
       <c r="CQ4" t="inlineStr"/>
+      <c r="CR4" t="inlineStr"/>
+      <c r="CS4" t="inlineStr"/>
+      <c r="CT4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1751,6 +1775,9 @@
       <c r="CO5" t="inlineStr"/>
       <c r="CP5" t="inlineStr"/>
       <c r="CQ5" t="inlineStr"/>
+      <c r="CR5" t="inlineStr"/>
+      <c r="CS5" t="inlineStr"/>
+      <c r="CT5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1968,6 +1995,9 @@
       <c r="CO6" t="inlineStr"/>
       <c r="CP6" t="inlineStr"/>
       <c r="CQ6" t="inlineStr"/>
+      <c r="CR6" t="inlineStr"/>
+      <c r="CS6" t="inlineStr"/>
+      <c r="CT6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2192,6 +2222,9 @@
       <c r="CO7" t="inlineStr"/>
       <c r="CP7" t="inlineStr"/>
       <c r="CQ7" t="inlineStr"/>
+      <c r="CR7" t="inlineStr"/>
+      <c r="CS7" t="inlineStr"/>
+      <c r="CT7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2411,6 +2444,9 @@
       <c r="CO8" t="inlineStr"/>
       <c r="CP8" t="inlineStr"/>
       <c r="CQ8" t="inlineStr"/>
+      <c r="CR8" t="inlineStr"/>
+      <c r="CS8" t="inlineStr"/>
+      <c r="CT8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2632,6 +2668,9 @@
       <c r="CO9" t="inlineStr"/>
       <c r="CP9" t="inlineStr"/>
       <c r="CQ9" t="inlineStr"/>
+      <c r="CR9" t="inlineStr"/>
+      <c r="CS9" t="inlineStr"/>
+      <c r="CT9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2853,6 +2892,9 @@
       <c r="CO10" t="inlineStr"/>
       <c r="CP10" t="inlineStr"/>
       <c r="CQ10" t="inlineStr"/>
+      <c r="CR10" t="inlineStr"/>
+      <c r="CS10" t="inlineStr"/>
+      <c r="CT10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3073,6 +3115,9 @@
       <c r="CO11" t="inlineStr"/>
       <c r="CP11" t="inlineStr"/>
       <c r="CQ11" t="inlineStr"/>
+      <c r="CR11" t="inlineStr"/>
+      <c r="CS11" t="inlineStr"/>
+      <c r="CT11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3297,6 +3342,9 @@
       <c r="CO12" t="inlineStr"/>
       <c r="CP12" t="inlineStr"/>
       <c r="CQ12" t="inlineStr"/>
+      <c r="CR12" t="inlineStr"/>
+      <c r="CS12" t="inlineStr"/>
+      <c r="CT12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3517,6 +3565,9 @@
       <c r="CO13" t="inlineStr"/>
       <c r="CP13" t="inlineStr"/>
       <c r="CQ13" t="inlineStr"/>
+      <c r="CR13" t="inlineStr"/>
+      <c r="CS13" t="inlineStr"/>
+      <c r="CT13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3726,6 +3777,9 @@
       <c r="CO14" t="inlineStr"/>
       <c r="CP14" t="inlineStr"/>
       <c r="CQ14" t="inlineStr"/>
+      <c r="CR14" t="inlineStr"/>
+      <c r="CS14" t="inlineStr"/>
+      <c r="CT14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3944,6 +3998,9 @@
       <c r="CO15" t="inlineStr"/>
       <c r="CP15" t="inlineStr"/>
       <c r="CQ15" t="inlineStr"/>
+      <c r="CR15" t="inlineStr"/>
+      <c r="CS15" t="inlineStr"/>
+      <c r="CT15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4158,6 +4215,9 @@
       <c r="CO16" t="inlineStr"/>
       <c r="CP16" t="inlineStr"/>
       <c r="CQ16" t="inlineStr"/>
+      <c r="CR16" t="inlineStr"/>
+      <c r="CS16" t="inlineStr"/>
+      <c r="CT16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
@@ -4295,6 +4355,9 @@
       <c r="CO17" t="inlineStr"/>
       <c r="CP17" t="inlineStr"/>
       <c r="CQ17" t="inlineStr"/>
+      <c r="CR17" t="inlineStr"/>
+      <c r="CS17" t="inlineStr"/>
+      <c r="CT17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4482,6 +4545,9 @@
       <c r="CO18" t="inlineStr"/>
       <c r="CP18" t="inlineStr"/>
       <c r="CQ18" t="inlineStr"/>
+      <c r="CR18" t="inlineStr"/>
+      <c r="CS18" t="inlineStr"/>
+      <c r="CT18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4675,6 +4741,9 @@
       <c r="CO19" t="inlineStr"/>
       <c r="CP19" t="inlineStr"/>
       <c r="CQ19" t="inlineStr"/>
+      <c r="CR19" t="inlineStr"/>
+      <c r="CS19" t="inlineStr"/>
+      <c r="CT19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4916,6 +4985,9 @@
       <c r="CO20" t="inlineStr"/>
       <c r="CP20" t="inlineStr"/>
       <c r="CQ20" t="inlineStr"/>
+      <c r="CR20" t="inlineStr"/>
+      <c r="CS20" t="inlineStr"/>
+      <c r="CT20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
@@ -5073,6 +5145,9 @@
       <c r="CO21" t="inlineStr"/>
       <c r="CP21" t="inlineStr"/>
       <c r="CQ21" t="inlineStr"/>
+      <c r="CR21" t="inlineStr"/>
+      <c r="CS21" t="inlineStr"/>
+      <c r="CT21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5322,6 +5397,9 @@
         <v>0</v>
       </c>
       <c r="CQ22" t="inlineStr"/>
+      <c r="CR22" t="inlineStr"/>
+      <c r="CS22" t="inlineStr"/>
+      <c r="CT22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5571,6 +5649,9 @@
         <v>0.9</v>
       </c>
       <c r="CQ23" t="inlineStr"/>
+      <c r="CR23" t="inlineStr"/>
+      <c r="CS23" t="inlineStr"/>
+      <c r="CT23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5820,6 +5901,9 @@
         <v>0</v>
       </c>
       <c r="CQ24" t="inlineStr"/>
+      <c r="CR24" t="inlineStr"/>
+      <c r="CS24" t="inlineStr"/>
+      <c r="CT24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6061,6 +6145,9 @@
         <v>0</v>
       </c>
       <c r="CQ25" t="inlineStr"/>
+      <c r="CR25" t="inlineStr"/>
+      <c r="CS25" t="inlineStr"/>
+      <c r="CT25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6094,15 +6181,11 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>99</t>
-        </is>
+      <c r="H26" t="n">
+        <v>5</v>
+      </c>
+      <c r="I26" t="n">
+        <v>99</v>
       </c>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
@@ -6120,87 +6203,55 @@
           <t>0,85x3,5mm</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
+      <c r="R26" t="n">
+        <v>9</v>
       </c>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="W26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="X26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Y26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Z26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AA26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AB26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AD26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AE26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AF26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AG26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AH26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AI26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="U26" t="n">
+        <v>1</v>
+      </c>
+      <c r="V26" t="n">
+        <v>1</v>
+      </c>
+      <c r="W26" t="n">
+        <v>1</v>
+      </c>
+      <c r="X26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI26" t="n">
+        <v>1</v>
       </c>
       <c r="AJ26" t="inlineStr">
         <is>
@@ -6297,47 +6348,786 @@
         <v>0</v>
       </c>
       <c r="CH26" t="inlineStr"/>
-      <c r="CI26" t="inlineStr">
+      <c r="CI26" t="n">
+        <v>1</v>
+      </c>
+      <c r="CJ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK26" t="n">
+        <v>1</v>
+      </c>
+      <c r="CL26" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM26" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN26" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO26" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP26" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ26" t="inlineStr"/>
+      <c r="CR26" t="inlineStr"/>
+      <c r="CS26" t="inlineStr"/>
+      <c r="CT26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2025-01-15</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>TESTE_BUG_RETROATIVO</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Dr. Daniel</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Alice</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>3</v>
+      </c>
+      <c r="I27" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1500</v>
+      </c>
+      <c r="K27" t="n">
+        <v>45</v>
+      </c>
+      <c r="L27" t="n">
+        <v>500</v>
+      </c>
+      <c r="M27" t="n">
+        <v>200</v>
+      </c>
+      <c r="N27" t="n">
+        <v>400</v>
+      </c>
+      <c r="O27" t="n">
+        <v>400</v>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>0,85x3,5mm</t>
+        </is>
+      </c>
+      <c r="R27" t="n">
+        <v>20</v>
+      </c>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="n">
+        <v>10</v>
+      </c>
+      <c r="V27" t="n">
+        <v>500</v>
+      </c>
+      <c r="W27" t="n">
+        <v>600</v>
+      </c>
+      <c r="X27" t="n">
+        <v>10</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>500</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>600</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB27" t="n">
+        <v>500</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>600</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>500</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>600</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK27" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL27" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM27" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN27" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO27" t="inlineStr"/>
+      <c r="AP27" t="inlineStr"/>
+      <c r="AQ27" t="inlineStr"/>
+      <c r="AR27" t="inlineStr"/>
+      <c r="AS27" t="inlineStr"/>
+      <c r="AT27" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU27" t="inlineStr"/>
+      <c r="AV27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX27" t="inlineStr"/>
+      <c r="AY27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA27" t="inlineStr"/>
+      <c r="BB27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD27" t="inlineStr"/>
+      <c r="BE27" t="inlineStr"/>
+      <c r="BF27" t="inlineStr"/>
+      <c r="BG27" t="inlineStr"/>
+      <c r="BH27" t="inlineStr"/>
+      <c r="BI27" t="inlineStr"/>
+      <c r="BJ27" t="inlineStr"/>
+      <c r="BK27" t="inlineStr"/>
+      <c r="BL27" t="inlineStr"/>
+      <c r="BM27" t="inlineStr"/>
+      <c r="BN27" t="inlineStr"/>
+      <c r="BO27" t="inlineStr"/>
+      <c r="BP27" t="inlineStr"/>
+      <c r="BQ27" t="inlineStr"/>
+      <c r="BR27" t="inlineStr"/>
+      <c r="BS27" t="inlineStr"/>
+      <c r="BT27" t="inlineStr"/>
+      <c r="BU27" t="inlineStr"/>
+      <c r="BV27" t="inlineStr"/>
+      <c r="BW27" t="inlineStr"/>
+      <c r="BX27" t="inlineStr"/>
+      <c r="BY27" t="inlineStr"/>
+      <c r="BZ27" t="inlineStr"/>
+      <c r="CA27" t="inlineStr"/>
+      <c r="CB27" t="inlineStr"/>
+      <c r="CC27" t="inlineStr"/>
+      <c r="CD27" t="inlineStr"/>
+      <c r="CE27" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="CF27" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG27" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH27" t="inlineStr"/>
+      <c r="CI27" t="inlineStr"/>
+      <c r="CJ27" t="inlineStr"/>
+      <c r="CK27" t="inlineStr"/>
+      <c r="CL27" t="inlineStr"/>
+      <c r="CM27" t="inlineStr"/>
+      <c r="CN27" t="inlineStr"/>
+      <c r="CO27" t="inlineStr"/>
+      <c r="CP27" t="inlineStr"/>
+      <c r="CQ27" t="inlineStr"/>
+      <c r="CR27" t="inlineStr">
+        <is>
+          <t>FUE</t>
+        </is>
+      </c>
+      <c r="CS27" t="inlineStr">
+        <is>
+          <t>DHI</t>
+        </is>
+      </c>
+      <c r="CT27" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2025-01-15</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>TESTE_BUG_RETROATIVO_DIFERENTE</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Dr. Daniel</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Alice</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>3</v>
+      </c>
+      <c r="I28" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1500</v>
+      </c>
+      <c r="K28" t="n">
+        <v>45</v>
+      </c>
+      <c r="L28" t="n">
+        <v>500</v>
+      </c>
+      <c r="M28" t="n">
+        <v>200</v>
+      </c>
+      <c r="N28" t="n">
+        <v>400</v>
+      </c>
+      <c r="O28" t="n">
+        <v>400</v>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>0,85x3,5mm</t>
+        </is>
+      </c>
+      <c r="R28" t="n">
+        <v>20</v>
+      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="n">
+        <v>10</v>
+      </c>
+      <c r="V28" t="n">
+        <v>500</v>
+      </c>
+      <c r="W28" t="n">
+        <v>600</v>
+      </c>
+      <c r="X28" t="n">
+        <v>10</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>500</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>600</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB28" t="n">
+        <v>500</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>600</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>500</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>600</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK28" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL28" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM28" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN28" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO28" t="inlineStr"/>
+      <c r="AP28" t="inlineStr"/>
+      <c r="AQ28" t="inlineStr"/>
+      <c r="AR28" t="inlineStr"/>
+      <c r="AS28" t="inlineStr"/>
+      <c r="AT28" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU28" t="inlineStr"/>
+      <c r="AV28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX28" t="inlineStr"/>
+      <c r="AY28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA28" t="inlineStr"/>
+      <c r="BB28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD28" t="inlineStr"/>
+      <c r="BE28" t="inlineStr"/>
+      <c r="BF28" t="inlineStr"/>
+      <c r="BG28" t="inlineStr"/>
+      <c r="BH28" t="inlineStr"/>
+      <c r="BI28" t="inlineStr"/>
+      <c r="BJ28" t="inlineStr"/>
+      <c r="BK28" t="inlineStr"/>
+      <c r="BL28" t="inlineStr"/>
+      <c r="BM28" t="inlineStr"/>
+      <c r="BN28" t="inlineStr"/>
+      <c r="BO28" t="inlineStr"/>
+      <c r="BP28" t="inlineStr"/>
+      <c r="BQ28" t="inlineStr"/>
+      <c r="BR28" t="inlineStr"/>
+      <c r="BS28" t="inlineStr"/>
+      <c r="BT28" t="inlineStr"/>
+      <c r="BU28" t="inlineStr"/>
+      <c r="BV28" t="inlineStr"/>
+      <c r="BW28" t="inlineStr"/>
+      <c r="BX28" t="inlineStr"/>
+      <c r="BY28" t="inlineStr"/>
+      <c r="BZ28" t="inlineStr"/>
+      <c r="CA28" t="inlineStr"/>
+      <c r="CB28" t="inlineStr"/>
+      <c r="CC28" t="inlineStr"/>
+      <c r="CD28" t="inlineStr"/>
+      <c r="CE28" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="CF28" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG28" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH28" t="inlineStr"/>
+      <c r="CI28" t="inlineStr"/>
+      <c r="CJ28" t="inlineStr"/>
+      <c r="CK28" t="inlineStr"/>
+      <c r="CL28" t="inlineStr"/>
+      <c r="CM28" t="inlineStr"/>
+      <c r="CN28" t="inlineStr"/>
+      <c r="CO28" t="inlineStr"/>
+      <c r="CP28" t="inlineStr"/>
+      <c r="CQ28" t="inlineStr"/>
+      <c r="CR28" t="inlineStr">
+        <is>
+          <t>FUE</t>
+        </is>
+      </c>
+      <c r="CS28" t="inlineStr">
+        <is>
+          <t>DHI</t>
+        </is>
+      </c>
+      <c r="CT28" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2025-01-15</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>TESTE_NOME_CURTO</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Dr. Daniel</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Alice</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>0,85x3,5mm</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="AF29" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="AG29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AH29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AI29" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="CJ26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="CK26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="CL26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="CM26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="CN26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="CO26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="CP26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="CQ26" t="inlineStr"/>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AK29" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL29" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM29" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN29" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO29" t="inlineStr"/>
+      <c r="AP29" t="inlineStr"/>
+      <c r="AQ29" t="inlineStr"/>
+      <c r="AR29" t="inlineStr"/>
+      <c r="AS29" t="inlineStr"/>
+      <c r="AT29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AU29" t="inlineStr"/>
+      <c r="AV29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX29" t="inlineStr"/>
+      <c r="AY29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA29" t="inlineStr"/>
+      <c r="BB29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD29" t="inlineStr"/>
+      <c r="BE29" t="inlineStr"/>
+      <c r="BF29" t="inlineStr"/>
+      <c r="BG29" t="inlineStr"/>
+      <c r="BH29" t="inlineStr"/>
+      <c r="BI29" t="inlineStr"/>
+      <c r="BJ29" t="inlineStr"/>
+      <c r="BK29" t="inlineStr"/>
+      <c r="BL29" t="inlineStr"/>
+      <c r="BM29" t="inlineStr"/>
+      <c r="BN29" t="inlineStr"/>
+      <c r="BO29" t="inlineStr"/>
+      <c r="BP29" t="inlineStr"/>
+      <c r="BQ29" t="inlineStr"/>
+      <c r="BR29" t="inlineStr"/>
+      <c r="BS29" t="inlineStr"/>
+      <c r="BT29" t="inlineStr"/>
+      <c r="BU29" t="inlineStr"/>
+      <c r="BV29" t="inlineStr"/>
+      <c r="BW29" t="inlineStr"/>
+      <c r="BX29" t="inlineStr"/>
+      <c r="BY29" t="inlineStr"/>
+      <c r="BZ29" t="inlineStr"/>
+      <c r="CA29" t="inlineStr"/>
+      <c r="CB29" t="inlineStr"/>
+      <c r="CC29" t="inlineStr"/>
+      <c r="CD29" t="inlineStr"/>
+      <c r="CE29" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="CF29" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG29" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH29" t="inlineStr"/>
+      <c r="CI29" t="inlineStr"/>
+      <c r="CJ29" t="inlineStr"/>
+      <c r="CK29" t="inlineStr"/>
+      <c r="CL29" t="inlineStr"/>
+      <c r="CM29" t="inlineStr"/>
+      <c r="CN29" t="inlineStr"/>
+      <c r="CO29" t="inlineStr"/>
+      <c r="CP29" t="inlineStr"/>
+      <c r="CQ29" t="inlineStr"/>
+      <c r="CR29" t="inlineStr">
+        <is>
+          <t>FUE</t>
+        </is>
+      </c>
+      <c r="CS29" t="inlineStr">
+        <is>
+          <t>DHI</t>
+        </is>
+      </c>
+      <c r="CT29" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>